<commit_message>
Unify shared scorecards and label incomplete round evidence
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12534" uniqueCount="2684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12579" uniqueCount="2687">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 13:38 BST</t>
+    <t>Snapshot: 07 September 2026, 13:42 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6528,6 +6528,15 @@
   </si>
   <si>
     <t>Shared round identity and scope</t>
+  </si>
+  <si>
+    <t>Both surfaces reuse full public scorecard, named owner/date/current limited scope, recorded partial counts/totals, row headers and pinned identity. Differential hidden unless valid complete9/18card; calculation unchanged. Dedicated safe404/loading/error recovery. shared-round-browser.log1PASS6.5s all12 surface/viewports,18rows/manualputts/fullrounddetails/read-only/noindex/nooverflow/noerrors; revocation removes data. Types/lint pass.</t>
+  </si>
+  <si>
+    <t>Same complete labelled horizontal scorecard with pinned hole identity and all existing allowed fields, full round details and public navigation.390/360/1023 checked on both surfaces;390 screenshot inspected. No private-app controls.</t>
+  </si>
+  <si>
+    <t>Backend DTO still calculates differential for partial cards; presentation suppression is not service fix (shared-round-partial.test.ts documented intentional failure). Full complete/empty/malformed/service-error browser matrix, keyboard table scroll, screen reader/native zoom/themes/physical touch outstanding. Access backend test separately verifies expired/revoked/wrong owner. Paid advanced examples unavailable; local semantic alternatives.</t>
   </si>
   <si>
     <t>Only the token-authorised frozen/current scope supported by the existing link is exposed.</t>
@@ -8245,8 +8254,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L474" totalsRowShown="0">
-  <autoFilter ref="A1:L474"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L477" totalsRowShown="0">
+  <autoFilter ref="A1:L477"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8640,11 +8649,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8679,11 +8688,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -26811,16 +26820,25 @@
         <v>42</v>
       </c>
       <c r="E475" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F475" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G475" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="H475" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="I475" s="4" t="s">
+        <v>2171</v>
       </c>
       <c r="J475" s="4" t="s">
-        <v>2169</v>
+        <v>2172</v>
       </c>
       <c r="K475" s="4" t="s">
-        <v>2170</v>
+        <v>2173</v>
       </c>
       <c r="L475" s="6" t="s">
         <v>39</v>
@@ -26828,28 +26846,37 @@
     </row>
     <row r="476" spans="1:12" ht="72" customHeight="1">
       <c r="A476" s="4" t="s">
-        <v>2171</v>
+        <v>2174</v>
       </c>
       <c r="B476" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C476" s="4" t="s">
-        <v>2172</v>
+        <v>2175</v>
       </c>
       <c r="D476" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E476" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F476" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G476" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="H476" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="I476" s="4" t="s">
+        <v>2171</v>
       </c>
       <c r="J476" s="4" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K476" s="4" t="s">
         <v>2173</v>
-      </c>
-      <c r="K476" s="4" t="s">
-        <v>2170</v>
       </c>
       <c r="L476" s="6" t="s">
         <v>88</v>
@@ -26857,28 +26884,37 @@
     </row>
     <row r="477" spans="1:12" ht="72" customHeight="1">
       <c r="A477" s="4" t="s">
-        <v>2174</v>
+        <v>2177</v>
       </c>
       <c r="B477" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C477" s="4" t="s">
-        <v>2175</v>
+        <v>2178</v>
       </c>
       <c r="D477" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E477" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F477" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G477" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="H477" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="I477" s="4" t="s">
+        <v>2171</v>
       </c>
       <c r="J477" s="4" t="s">
-        <v>2176</v>
+        <v>2179</v>
       </c>
       <c r="K477" s="4" t="s">
-        <v>2170</v>
+        <v>2173</v>
       </c>
       <c r="L477" s="6" t="s">
         <v>110</v>
@@ -26886,13 +26922,13 @@
     </row>
     <row r="478" spans="1:12" ht="72" customHeight="1">
       <c r="A478" s="4" t="s">
-        <v>2177</v>
+        <v>2180</v>
       </c>
       <c r="B478" s="4" t="s">
-        <v>2178</v>
+        <v>2181</v>
       </c>
       <c r="C478" s="4" t="s">
-        <v>2179</v>
+        <v>2182</v>
       </c>
       <c r="D478" s="4" t="s">
         <v>42</v>
@@ -26904,10 +26940,10 @@
         <v>9</v>
       </c>
       <c r="J478" s="4" t="s">
-        <v>2180</v>
+        <v>2183</v>
       </c>
       <c r="K478" s="4" t="s">
-        <v>2181</v>
+        <v>2184</v>
       </c>
       <c r="L478" s="6" t="s">
         <v>39</v>
@@ -26915,13 +26951,13 @@
     </row>
     <row r="479" spans="1:12" ht="72" customHeight="1">
       <c r="A479" s="4" t="s">
-        <v>2182</v>
+        <v>2185</v>
       </c>
       <c r="B479" s="4" t="s">
-        <v>2178</v>
+        <v>2181</v>
       </c>
       <c r="C479" s="4" t="s">
-        <v>2183</v>
+        <v>2186</v>
       </c>
       <c r="D479" s="4" t="s">
         <v>42</v>
@@ -26933,10 +26969,10 @@
         <v>9</v>
       </c>
       <c r="J479" s="4" t="s">
-        <v>2184</v>
+        <v>2187</v>
       </c>
       <c r="K479" s="4" t="s">
-        <v>2185</v>
+        <v>2188</v>
       </c>
       <c r="L479" s="6" t="s">
         <v>95</v>
@@ -26944,13 +26980,13 @@
     </row>
     <row r="480" spans="1:12" ht="72" customHeight="1">
       <c r="A480" s="4" t="s">
-        <v>2186</v>
+        <v>2189</v>
       </c>
       <c r="B480" s="4" t="s">
-        <v>2178</v>
+        <v>2181</v>
       </c>
       <c r="C480" s="4" t="s">
-        <v>2187</v>
+        <v>2190</v>
       </c>
       <c r="D480" s="4" t="s">
         <v>42</v>
@@ -26962,10 +26998,10 @@
         <v>9</v>
       </c>
       <c r="J480" s="4" t="s">
-        <v>2188</v>
+        <v>2191</v>
       </c>
       <c r="K480" s="4" t="s">
-        <v>2189</v>
+        <v>2192</v>
       </c>
       <c r="L480" s="6" t="s">
         <v>110</v>
@@ -26973,13 +27009,13 @@
     </row>
     <row r="481" spans="1:12" ht="72" customHeight="1">
       <c r="A481" s="4" t="s">
-        <v>2190</v>
+        <v>2193</v>
       </c>
       <c r="B481" s="4" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="C481" s="4" t="s">
-        <v>2192</v>
+        <v>2195</v>
       </c>
       <c r="D481" s="4" t="s">
         <v>42</v>
@@ -26991,10 +27027,10 @@
         <v>9</v>
       </c>
       <c r="J481" s="4" t="s">
-        <v>2193</v>
+        <v>2196</v>
       </c>
       <c r="K481" s="4" t="s">
-        <v>2194</v>
+        <v>2197</v>
       </c>
       <c r="L481" s="6" t="s">
         <v>518</v>
@@ -27002,13 +27038,13 @@
     </row>
     <row r="482" spans="1:12" ht="72" customHeight="1">
       <c r="A482" s="4" t="s">
-        <v>2195</v>
+        <v>2198</v>
       </c>
       <c r="B482" s="4" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="C482" s="4" t="s">
-        <v>2196</v>
+        <v>2199</v>
       </c>
       <c r="D482" s="4" t="s">
         <v>42</v>
@@ -27020,10 +27056,10 @@
         <v>9</v>
       </c>
       <c r="J482" s="4" t="s">
-        <v>2197</v>
+        <v>2200</v>
       </c>
       <c r="K482" s="4" t="s">
-        <v>2198</v>
+        <v>2201</v>
       </c>
       <c r="L482" s="6" t="s">
         <v>307</v>
@@ -27031,13 +27067,13 @@
     </row>
     <row r="483" spans="1:12" ht="72" customHeight="1">
       <c r="A483" s="4" t="s">
-        <v>2199</v>
+        <v>2202</v>
       </c>
       <c r="B483" s="4" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="C483" s="4" t="s">
-        <v>2200</v>
+        <v>2203</v>
       </c>
       <c r="D483" s="4" t="s">
         <v>42</v>
@@ -27049,10 +27085,10 @@
         <v>9</v>
       </c>
       <c r="J483" s="4" t="s">
-        <v>2201</v>
+        <v>2204</v>
       </c>
       <c r="K483" s="4" t="s">
-        <v>2202</v>
+        <v>2205</v>
       </c>
       <c r="L483" s="6" t="s">
         <v>110</v>
@@ -27060,13 +27096,13 @@
     </row>
     <row r="484" spans="1:12" ht="72" customHeight="1">
       <c r="A484" s="4" t="s">
-        <v>2203</v>
+        <v>2206</v>
       </c>
       <c r="B484" s="4" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="C484" s="4" t="s">
-        <v>2205</v>
+        <v>2208</v>
       </c>
       <c r="D484" s="4" t="s">
         <v>32</v>
@@ -27078,10 +27114,10 @@
         <v>9</v>
       </c>
       <c r="J484" s="4" t="s">
-        <v>2206</v>
+        <v>2209</v>
       </c>
       <c r="K484" s="4" t="s">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="L484" s="6" t="s">
         <v>165</v>
@@ -27089,13 +27125,13 @@
     </row>
     <row r="485" spans="1:12" ht="72" customHeight="1">
       <c r="A485" s="4" t="s">
-        <v>2208</v>
+        <v>2211</v>
       </c>
       <c r="B485" s="4" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="C485" s="4" t="s">
-        <v>2209</v>
+        <v>2212</v>
       </c>
       <c r="D485" s="4" t="s">
         <v>32</v>
@@ -27107,10 +27143,10 @@
         <v>9</v>
       </c>
       <c r="J485" s="4" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="K485" s="4" t="s">
-        <v>2211</v>
+        <v>2214</v>
       </c>
       <c r="L485" s="6" t="s">
         <v>110</v>
@@ -27118,13 +27154,13 @@
     </row>
     <row r="486" spans="1:12" ht="72" customHeight="1">
       <c r="A486" s="4" t="s">
-        <v>2212</v>
+        <v>2215</v>
       </c>
       <c r="B486" s="4" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="C486" s="4" t="s">
-        <v>2214</v>
+        <v>2217</v>
       </c>
       <c r="D486" s="4" t="s">
         <v>42</v>
@@ -27136,10 +27172,10 @@
         <v>9</v>
       </c>
       <c r="J486" s="4" t="s">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="K486" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="L486" s="6" t="s">
         <v>165</v>
@@ -27147,13 +27183,13 @@
     </row>
     <row r="487" spans="1:12" ht="72" customHeight="1">
       <c r="A487" s="4" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="B487" s="4" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="C487" s="4" t="s">
-        <v>2218</v>
+        <v>2221</v>
       </c>
       <c r="D487" s="4" t="s">
         <v>42</v>
@@ -27165,10 +27201,10 @@
         <v>9</v>
       </c>
       <c r="J487" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="K487" s="4" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="L487" s="6" t="s">
         <v>165</v>
@@ -27176,13 +27212,13 @@
     </row>
     <row r="488" spans="1:12" ht="72" customHeight="1">
       <c r="A488" s="4" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="B488" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="C488" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D488" s="4" t="s">
         <v>42</v>
@@ -27194,10 +27230,10 @@
         <v>9</v>
       </c>
       <c r="J488" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K488" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="L488" s="6" t="s">
         <v>141</v>
@@ -27205,13 +27241,13 @@
     </row>
     <row r="489" spans="1:12" ht="72" customHeight="1">
       <c r="A489" s="4" t="s">
+        <v>2229</v>
+      </c>
+      <c r="B489" s="4" t="s">
+        <v>2230</v>
+      </c>
+      <c r="C489" s="4" t="s">
         <v>2226</v>
-      </c>
-      <c r="B489" s="4" t="s">
-        <v>2227</v>
-      </c>
-      <c r="C489" s="4" t="s">
-        <v>2223</v>
       </c>
       <c r="D489" s="4" t="s">
         <v>42</v>
@@ -27223,10 +27259,10 @@
         <v>9</v>
       </c>
       <c r="J489" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27234,13 +27270,13 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="C490" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D490" s="4" t="s">
         <v>42</v>
@@ -27252,10 +27288,10 @@
         <v>9</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27263,13 +27299,13 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="C491" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D491" s="4" t="s">
         <v>42</v>
@@ -27281,10 +27317,10 @@
         <v>9</v>
       </c>
       <c r="J491" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27292,13 +27328,13 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="C492" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D492" s="4" t="s">
         <v>42</v>
@@ -27310,10 +27346,10 @@
         <v>9</v>
       </c>
       <c r="J492" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27321,13 +27357,13 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C493" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D493" s="4" t="s">
         <v>42</v>
@@ -27339,10 +27375,10 @@
         <v>9</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -27873,7 +27909,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L474"/>
+  <dimension ref="A1:L477"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -45888,8 +45924,122 @@
         <v>47</v>
       </c>
     </row>
+    <row r="475" spans="1:12" ht="72" customHeight="1">
+      <c r="A475" s="4" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B475" s="4" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C475" s="4" t="s">
+        <v>2168</v>
+      </c>
+      <c r="D475" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E475" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F475" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G475" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="H475" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="I475" s="4" t="s">
+        <v>2171</v>
+      </c>
+      <c r="J475" s="4" t="s">
+        <v>2172</v>
+      </c>
+      <c r="K475" s="4" t="s">
+        <v>2173</v>
+      </c>
+      <c r="L475" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="476" spans="1:12" ht="72" customHeight="1">
+      <c r="A476" s="4" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B476" s="4" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C476" s="4" t="s">
+        <v>2175</v>
+      </c>
+      <c r="D476" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E476" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F476" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G476" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="H476" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="I476" s="4" t="s">
+        <v>2171</v>
+      </c>
+      <c r="J476" s="4" t="s">
+        <v>2176</v>
+      </c>
+      <c r="K476" s="4" t="s">
+        <v>2173</v>
+      </c>
+      <c r="L476" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="477" spans="1:12" ht="72" customHeight="1">
+      <c r="A477" s="4" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B477" s="4" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C477" s="4" t="s">
+        <v>2178</v>
+      </c>
+      <c r="D477" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E477" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F477" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G477" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="H477" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="I477" s="4" t="s">
+        <v>2171</v>
+      </c>
+      <c r="J477" s="4" t="s">
+        <v>2179</v>
+      </c>
+      <c r="K477" s="4" t="s">
+        <v>2173</v>
+      </c>
+      <c r="L477" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F474">
+  <conditionalFormatting sqref="E2:F477">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -46380,11 +46530,14 @@
     <hyperlink ref="L472" r:id="rId471"/>
     <hyperlink ref="L473" r:id="rId472"/>
     <hyperlink ref="L474" r:id="rId473"/>
+    <hyperlink ref="L475" r:id="rId474"/>
+    <hyperlink ref="L476" r:id="rId475"/>
+    <hyperlink ref="L477" r:id="rId476"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId474"/>
+    <tablePart r:id="rId477"/>
   </tableParts>
 </worksheet>
 </file>
@@ -46401,3128 +46554,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2440</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2441</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2289</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2442</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2257</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2436</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2437</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2438</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2286</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2439</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2254</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2433</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2434</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2289</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2588</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2257</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2584</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2286</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2585</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2254</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2581</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2635</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2636</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2314</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2637</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2631</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2638</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2632</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2633</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2311</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2634</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2628</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2635</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2629</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2650</v>
+        <v>2653</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>2178</v>
+        <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>2198</v>
+        <v>2201</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>2211</v>
+        <v>2214</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
+        <v>2677</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2230</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>2678</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>2231</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>2674</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>2227</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
+        <v>2229</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>2257</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>2675</v>
       </c>
-      <c r="D95" s="4" t="s">
-        <v>2228</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>2671</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>2226</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>2254</v>
-      </c>
-      <c r="H95" s="4" t="s">
-        <v>2672</v>
-      </c>
       <c r="I95" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2679</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2233</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2680</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2234</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2674</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2232</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2257</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2675</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2676</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2230</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2677</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2231</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2671</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2229</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2254</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2672</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2673</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expose shared Course Twin scope above preserved responsive runtime
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12579" uniqueCount="2687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12624" uniqueCount="2690">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 13:42 BST</t>
+    <t>Snapshot: 07 September 2026, 13:46 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6570,6 +6570,15 @@
   </si>
   <si>
     <t>Shared twin identity and access scope</t>
+  </si>
+  <si>
+    <t>Shared Twin visible compact title/scope/public exit, canonical readOnly replay renderer preserved; noindex metadata and separate unavailable/loading/service-error boundaries. shared-twin-browser-final.log1PASS2.1s six sizes canonical2D fallback/hole selection/no private mutations/no overflow/errors. Page handoff2unitPASS; types/lint clean.</t>
+  </si>
+  <si>
+    <t>Normal-flow title and limited public scope remain visible above usable runtime;390/360/1023 fallback Previous/selectedhole/exit checked,390 screenshot reviewed. Existing geometry/reconstructed-flight labels and full touch controls preserved.</t>
+  </si>
+  <si>
+    <t>Actual shared app route visual run, measured-shot replay and liveWebGL/context-loss/3D toggle/device/reduced-motion matrix, screen-reader/native zoom/themes outstanding. Isolated scene intentionally stubbed; real canonical2D controls used. Token backend regression1PASS validates revoked/expired/foreignowner/wrongtype rejected before manifest/replay loading. Paid advanced examples unavailable; local accessible shell.</t>
   </si>
   <si>
     <t>Token permissions remain enforced and private runtime controls are absent.</t>
@@ -8254,8 +8263,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L477" totalsRowShown="0">
-  <autoFilter ref="A1:L477"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L480" totalsRowShown="0">
+  <autoFilter ref="A1:L480"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8649,11 +8658,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8688,11 +8697,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -26934,16 +26943,25 @@
         <v>42</v>
       </c>
       <c r="E478" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F478" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G478" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="H478" s="4" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I478" s="4" t="s">
+        <v>2185</v>
       </c>
       <c r="J478" s="4" t="s">
-        <v>2183</v>
+        <v>2186</v>
       </c>
       <c r="K478" s="4" t="s">
-        <v>2184</v>
+        <v>2187</v>
       </c>
       <c r="L478" s="6" t="s">
         <v>39</v>
@@ -26951,28 +26969,37 @@
     </row>
     <row r="479" spans="1:12" ht="72" customHeight="1">
       <c r="A479" s="4" t="s">
-        <v>2185</v>
+        <v>2188</v>
       </c>
       <c r="B479" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C479" s="4" t="s">
-        <v>2186</v>
+        <v>2189</v>
       </c>
       <c r="D479" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E479" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F479" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G479" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="H479" s="4" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I479" s="4" t="s">
+        <v>2185</v>
       </c>
       <c r="J479" s="4" t="s">
-        <v>2187</v>
+        <v>2190</v>
       </c>
       <c r="K479" s="4" t="s">
-        <v>2188</v>
+        <v>2191</v>
       </c>
       <c r="L479" s="6" t="s">
         <v>95</v>
@@ -26980,28 +27007,37 @@
     </row>
     <row r="480" spans="1:12" ht="72" customHeight="1">
       <c r="A480" s="4" t="s">
-        <v>2189</v>
+        <v>2192</v>
       </c>
       <c r="B480" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C480" s="4" t="s">
-        <v>2190</v>
+        <v>2193</v>
       </c>
       <c r="D480" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E480" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F480" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G480" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="H480" s="4" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I480" s="4" t="s">
+        <v>2185</v>
       </c>
       <c r="J480" s="4" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="K480" s="4" t="s">
-        <v>2192</v>
+        <v>2195</v>
       </c>
       <c r="L480" s="6" t="s">
         <v>110</v>
@@ -27009,13 +27045,13 @@
     </row>
     <row r="481" spans="1:12" ht="72" customHeight="1">
       <c r="A481" s="4" t="s">
-        <v>2193</v>
+        <v>2196</v>
       </c>
       <c r="B481" s="4" t="s">
-        <v>2194</v>
+        <v>2197</v>
       </c>
       <c r="C481" s="4" t="s">
-        <v>2195</v>
+        <v>2198</v>
       </c>
       <c r="D481" s="4" t="s">
         <v>42</v>
@@ -27027,10 +27063,10 @@
         <v>9</v>
       </c>
       <c r="J481" s="4" t="s">
-        <v>2196</v>
+        <v>2199</v>
       </c>
       <c r="K481" s="4" t="s">
-        <v>2197</v>
+        <v>2200</v>
       </c>
       <c r="L481" s="6" t="s">
         <v>518</v>
@@ -27038,13 +27074,13 @@
     </row>
     <row r="482" spans="1:12" ht="72" customHeight="1">
       <c r="A482" s="4" t="s">
-        <v>2198</v>
+        <v>2201</v>
       </c>
       <c r="B482" s="4" t="s">
-        <v>2194</v>
+        <v>2197</v>
       </c>
       <c r="C482" s="4" t="s">
-        <v>2199</v>
+        <v>2202</v>
       </c>
       <c r="D482" s="4" t="s">
         <v>42</v>
@@ -27056,10 +27092,10 @@
         <v>9</v>
       </c>
       <c r="J482" s="4" t="s">
-        <v>2200</v>
+        <v>2203</v>
       </c>
       <c r="K482" s="4" t="s">
-        <v>2201</v>
+        <v>2204</v>
       </c>
       <c r="L482" s="6" t="s">
         <v>307</v>
@@ -27067,13 +27103,13 @@
     </row>
     <row r="483" spans="1:12" ht="72" customHeight="1">
       <c r="A483" s="4" t="s">
-        <v>2202</v>
+        <v>2205</v>
       </c>
       <c r="B483" s="4" t="s">
-        <v>2194</v>
+        <v>2197</v>
       </c>
       <c r="C483" s="4" t="s">
-        <v>2203</v>
+        <v>2206</v>
       </c>
       <c r="D483" s="4" t="s">
         <v>42</v>
@@ -27085,10 +27121,10 @@
         <v>9</v>
       </c>
       <c r="J483" s="4" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="K483" s="4" t="s">
-        <v>2205</v>
+        <v>2208</v>
       </c>
       <c r="L483" s="6" t="s">
         <v>110</v>
@@ -27096,13 +27132,13 @@
     </row>
     <row r="484" spans="1:12" ht="72" customHeight="1">
       <c r="A484" s="4" t="s">
-        <v>2206</v>
+        <v>2209</v>
       </c>
       <c r="B484" s="4" t="s">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="C484" s="4" t="s">
-        <v>2208</v>
+        <v>2211</v>
       </c>
       <c r="D484" s="4" t="s">
         <v>32</v>
@@ -27114,10 +27150,10 @@
         <v>9</v>
       </c>
       <c r="J484" s="4" t="s">
-        <v>2209</v>
+        <v>2212</v>
       </c>
       <c r="K484" s="4" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="L484" s="6" t="s">
         <v>165</v>
@@ -27125,13 +27161,13 @@
     </row>
     <row r="485" spans="1:12" ht="72" customHeight="1">
       <c r="A485" s="4" t="s">
-        <v>2211</v>
+        <v>2214</v>
       </c>
       <c r="B485" s="4" t="s">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="C485" s="4" t="s">
-        <v>2212</v>
+        <v>2215</v>
       </c>
       <c r="D485" s="4" t="s">
         <v>32</v>
@@ -27143,10 +27179,10 @@
         <v>9</v>
       </c>
       <c r="J485" s="4" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="K485" s="4" t="s">
-        <v>2214</v>
+        <v>2217</v>
       </c>
       <c r="L485" s="6" t="s">
         <v>110</v>
@@ -27154,13 +27190,13 @@
     </row>
     <row r="486" spans="1:12" ht="72" customHeight="1">
       <c r="A486" s="4" t="s">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="B486" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="C486" s="4" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="D486" s="4" t="s">
         <v>42</v>
@@ -27172,10 +27208,10 @@
         <v>9</v>
       </c>
       <c r="J486" s="4" t="s">
-        <v>2218</v>
+        <v>2221</v>
       </c>
       <c r="K486" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="L486" s="6" t="s">
         <v>165</v>
@@ -27183,13 +27219,13 @@
     </row>
     <row r="487" spans="1:12" ht="72" customHeight="1">
       <c r="A487" s="4" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="B487" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="C487" s="4" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="D487" s="4" t="s">
         <v>42</v>
@@ -27201,10 +27237,10 @@
         <v>9</v>
       </c>
       <c r="J487" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="K487" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="L487" s="6" t="s">
         <v>165</v>
@@ -27212,13 +27248,13 @@
     </row>
     <row r="488" spans="1:12" ht="72" customHeight="1">
       <c r="A488" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="B488" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="C488" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="D488" s="4" t="s">
         <v>42</v>
@@ -27230,10 +27266,10 @@
         <v>9</v>
       </c>
       <c r="J488" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K488" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="L488" s="6" t="s">
         <v>141</v>
@@ -27241,13 +27277,13 @@
     </row>
     <row r="489" spans="1:12" ht="72" customHeight="1">
       <c r="A489" s="4" t="s">
+        <v>2232</v>
+      </c>
+      <c r="B489" s="4" t="s">
+        <v>2233</v>
+      </c>
+      <c r="C489" s="4" t="s">
         <v>2229</v>
-      </c>
-      <c r="B489" s="4" t="s">
-        <v>2230</v>
-      </c>
-      <c r="C489" s="4" t="s">
-        <v>2226</v>
       </c>
       <c r="D489" s="4" t="s">
         <v>42</v>
@@ -27259,10 +27295,10 @@
         <v>9</v>
       </c>
       <c r="J489" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27270,13 +27306,13 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="C490" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="D490" s="4" t="s">
         <v>42</v>
@@ -27288,10 +27324,10 @@
         <v>9</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27299,13 +27335,13 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="C491" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="D491" s="4" t="s">
         <v>42</v>
@@ -27317,10 +27353,10 @@
         <v>9</v>
       </c>
       <c r="J491" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27328,13 +27364,13 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C492" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="D492" s="4" t="s">
         <v>42</v>
@@ -27346,10 +27382,10 @@
         <v>9</v>
       </c>
       <c r="J492" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27357,13 +27393,13 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C493" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="D493" s="4" t="s">
         <v>42</v>
@@ -27375,10 +27411,10 @@
         <v>9</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -27909,7 +27945,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L477"/>
+  <dimension ref="A1:L480"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46038,8 +46074,122 @@
         <v>110</v>
       </c>
     </row>
+    <row r="478" spans="1:12" ht="72" customHeight="1">
+      <c r="A478" s="4" t="s">
+        <v>2180</v>
+      </c>
+      <c r="B478" s="4" t="s">
+        <v>2181</v>
+      </c>
+      <c r="C478" s="4" t="s">
+        <v>2182</v>
+      </c>
+      <c r="D478" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E478" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F478" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G478" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="H478" s="4" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I478" s="4" t="s">
+        <v>2185</v>
+      </c>
+      <c r="J478" s="4" t="s">
+        <v>2186</v>
+      </c>
+      <c r="K478" s="4" t="s">
+        <v>2187</v>
+      </c>
+      <c r="L478" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="479" spans="1:12" ht="72" customHeight="1">
+      <c r="A479" s="4" t="s">
+        <v>2188</v>
+      </c>
+      <c r="B479" s="4" t="s">
+        <v>2181</v>
+      </c>
+      <c r="C479" s="4" t="s">
+        <v>2189</v>
+      </c>
+      <c r="D479" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E479" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F479" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G479" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="H479" s="4" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I479" s="4" t="s">
+        <v>2185</v>
+      </c>
+      <c r="J479" s="4" t="s">
+        <v>2190</v>
+      </c>
+      <c r="K479" s="4" t="s">
+        <v>2191</v>
+      </c>
+      <c r="L479" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="480" spans="1:12" ht="72" customHeight="1">
+      <c r="A480" s="4" t="s">
+        <v>2192</v>
+      </c>
+      <c r="B480" s="4" t="s">
+        <v>2181</v>
+      </c>
+      <c r="C480" s="4" t="s">
+        <v>2193</v>
+      </c>
+      <c r="D480" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E480" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F480" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G480" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="H480" s="4" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I480" s="4" t="s">
+        <v>2185</v>
+      </c>
+      <c r="J480" s="4" t="s">
+        <v>2194</v>
+      </c>
+      <c r="K480" s="4" t="s">
+        <v>2195</v>
+      </c>
+      <c r="L480" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F477">
+  <conditionalFormatting sqref="E2:F480">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -46533,11 +46683,14 @@
     <hyperlink ref="L475" r:id="rId474"/>
     <hyperlink ref="L476" r:id="rId475"/>
     <hyperlink ref="L477" r:id="rId476"/>
+    <hyperlink ref="L478" r:id="rId477"/>
+    <hyperlink ref="L479" r:id="rId478"/>
+    <hyperlink ref="L480" r:id="rId479"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId477"/>
+    <tablePart r:id="rId480"/>
   </tableParts>
 </worksheet>
 </file>
@@ -46554,3128 +46707,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2443</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2444</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2292</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2445</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2260</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2439</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2440</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2441</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2289</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2442</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2257</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2436</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2437</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2590</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2292</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2591</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2260</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2587</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2289</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2588</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2257</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2584</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2638</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2639</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2317</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2640</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2634</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2641</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2635</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2636</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2314</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2637</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2631</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2638</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2632</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2650</v>
+        <v>2653</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>2194</v>
+        <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>2201</v>
+        <v>2204</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>2214</v>
+        <v>2217</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
+        <v>2680</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2233</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>2681</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>2234</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>2677</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>2230</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
+        <v>2232</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>2260</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>2678</v>
       </c>
-      <c r="D95" s="4" t="s">
-        <v>2231</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>2674</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>2229</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>2257</v>
-      </c>
-      <c r="H95" s="4" t="s">
-        <v>2675</v>
-      </c>
       <c r="I95" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2682</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2236</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2683</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2237</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2677</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2235</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2260</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2678</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2679</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2233</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2680</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2234</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2674</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2232</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2257</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2675</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2676</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deliver full responsive shared reports with recoverable password access
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12624" uniqueCount="2690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12669" uniqueCount="2693">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 13:46 BST</t>
+    <t>Snapshot: 07 September 2026, 13:54 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6618,6 +6618,15 @@
   </si>
   <si>
     <t>Password-protected report gate</t>
+  </si>
+  <si>
+    <t>Unified full frozen report sections with selected scope/date, full-width layout, labelled scrollable pinned-identity evidence tables including units and raw quality. Stateful password retry retains input, show/hide, pending/inlineerrors, server validation/cookie retained. Dedicated404/error/loading/publicreturn. shared-report-browser-ready.log1PASS16.5s all12 surfaces/viewports actual synthetic report: no evidence before access, wrong-password retained, correct unlock, selected sections only, revocation hides data. Types/lint clean.</t>
+  </si>
+  <si>
+    <t>Same complete report evidence and accessible table regions on390/360/1023 both surfaces, natural wrapping/public navigation; password44pxcontrols and successful recovery same browser pass.390 report screenshot inspected. No summary substitute.</t>
+  </si>
+  <si>
+    <t>All12 optional evidence-section combinations, native software keyboard/safe-area/screen-reader/zoom/theme/fullservice-error states outstanding. Existing report/page.tsx concurrent view-history change remains unstaged and unclaimed in this UI commit. Action6unitPASS plus realDB access1PASS and history2PASS separately; mock cookies not physical-browser proof. Paid advanced examples unavailable; local accessible alternative.</t>
   </si>
   <si>
     <t>Password and token validation remain server-side; no report data appears before access is granted.</t>
@@ -8263,8 +8272,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L480" totalsRowShown="0">
-  <autoFilter ref="A1:L480"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L483" totalsRowShown="0">
+  <autoFilter ref="A1:L483"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8658,11 +8667,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8697,11 +8706,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -27057,16 +27066,25 @@
         <v>42</v>
       </c>
       <c r="E481" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F481" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G481" s="4" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H481" s="4" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I481" s="4" t="s">
+        <v>2201</v>
       </c>
       <c r="J481" s="4" t="s">
-        <v>2199</v>
+        <v>2202</v>
       </c>
       <c r="K481" s="4" t="s">
-        <v>2200</v>
+        <v>2203</v>
       </c>
       <c r="L481" s="6" t="s">
         <v>518</v>
@@ -27074,28 +27092,37 @@
     </row>
     <row r="482" spans="1:12" ht="72" customHeight="1">
       <c r="A482" s="4" t="s">
-        <v>2201</v>
+        <v>2204</v>
       </c>
       <c r="B482" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C482" s="4" t="s">
-        <v>2202</v>
+        <v>2205</v>
       </c>
       <c r="D482" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E482" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F482" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G482" s="4" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H482" s="4" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I482" s="4" t="s">
+        <v>2201</v>
       </c>
       <c r="J482" s="4" t="s">
-        <v>2203</v>
+        <v>2206</v>
       </c>
       <c r="K482" s="4" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="L482" s="6" t="s">
         <v>307</v>
@@ -27103,28 +27130,37 @@
     </row>
     <row r="483" spans="1:12" ht="72" customHeight="1">
       <c r="A483" s="4" t="s">
-        <v>2205</v>
+        <v>2208</v>
       </c>
       <c r="B483" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C483" s="4" t="s">
-        <v>2206</v>
+        <v>2209</v>
       </c>
       <c r="D483" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E483" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F483" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G483" s="4" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H483" s="4" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I483" s="4" t="s">
+        <v>2201</v>
       </c>
       <c r="J483" s="4" t="s">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="K483" s="4" t="s">
-        <v>2208</v>
+        <v>2211</v>
       </c>
       <c r="L483" s="6" t="s">
         <v>110</v>
@@ -27132,13 +27168,13 @@
     </row>
     <row r="484" spans="1:12" ht="72" customHeight="1">
       <c r="A484" s="4" t="s">
-        <v>2209</v>
+        <v>2212</v>
       </c>
       <c r="B484" s="4" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="C484" s="4" t="s">
-        <v>2211</v>
+        <v>2214</v>
       </c>
       <c r="D484" s="4" t="s">
         <v>32</v>
@@ -27150,10 +27186,10 @@
         <v>9</v>
       </c>
       <c r="J484" s="4" t="s">
-        <v>2212</v>
+        <v>2215</v>
       </c>
       <c r="K484" s="4" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="L484" s="6" t="s">
         <v>165</v>
@@ -27161,13 +27197,13 @@
     </row>
     <row r="485" spans="1:12" ht="72" customHeight="1">
       <c r="A485" s="4" t="s">
-        <v>2214</v>
+        <v>2217</v>
       </c>
       <c r="B485" s="4" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="C485" s="4" t="s">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="D485" s="4" t="s">
         <v>32</v>
@@ -27179,10 +27215,10 @@
         <v>9</v>
       </c>
       <c r="J485" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="K485" s="4" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="L485" s="6" t="s">
         <v>110</v>
@@ -27190,13 +27226,13 @@
     </row>
     <row r="486" spans="1:12" ht="72" customHeight="1">
       <c r="A486" s="4" t="s">
-        <v>2218</v>
+        <v>2221</v>
       </c>
       <c r="B486" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="C486" s="4" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="D486" s="4" t="s">
         <v>42</v>
@@ -27208,10 +27244,10 @@
         <v>9</v>
       </c>
       <c r="J486" s="4" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="K486" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="L486" s="6" t="s">
         <v>165</v>
@@ -27219,13 +27255,13 @@
     </row>
     <row r="487" spans="1:12" ht="72" customHeight="1">
       <c r="A487" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="B487" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="C487" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="D487" s="4" t="s">
         <v>42</v>
@@ -27237,10 +27273,10 @@
         <v>9</v>
       </c>
       <c r="J487" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="K487" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="L487" s="6" t="s">
         <v>165</v>
@@ -27248,13 +27284,13 @@
     </row>
     <row r="488" spans="1:12" ht="72" customHeight="1">
       <c r="A488" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="B488" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="C488" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="D488" s="4" t="s">
         <v>42</v>
@@ -27266,10 +27302,10 @@
         <v>9</v>
       </c>
       <c r="J488" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="K488" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="L488" s="6" t="s">
         <v>141</v>
@@ -27277,13 +27313,13 @@
     </row>
     <row r="489" spans="1:12" ht="72" customHeight="1">
       <c r="A489" s="4" t="s">
+        <v>2235</v>
+      </c>
+      <c r="B489" s="4" t="s">
+        <v>2236</v>
+      </c>
+      <c r="C489" s="4" t="s">
         <v>2232</v>
-      </c>
-      <c r="B489" s="4" t="s">
-        <v>2233</v>
-      </c>
-      <c r="C489" s="4" t="s">
-        <v>2229</v>
       </c>
       <c r="D489" s="4" t="s">
         <v>42</v>
@@ -27295,10 +27331,10 @@
         <v>9</v>
       </c>
       <c r="J489" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27306,13 +27342,13 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="C490" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="D490" s="4" t="s">
         <v>42</v>
@@ -27324,10 +27360,10 @@
         <v>9</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27335,13 +27371,13 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C491" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="D491" s="4" t="s">
         <v>42</v>
@@ -27353,10 +27389,10 @@
         <v>9</v>
       </c>
       <c r="J491" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27364,13 +27400,13 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C492" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="D492" s="4" t="s">
         <v>42</v>
@@ -27382,10 +27418,10 @@
         <v>9</v>
       </c>
       <c r="J492" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27393,13 +27429,13 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C493" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="D493" s="4" t="s">
         <v>42</v>
@@ -27411,10 +27447,10 @@
         <v>9</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -27945,7 +27981,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L480"/>
+  <dimension ref="A1:L483"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46188,8 +46224,122 @@
         <v>110</v>
       </c>
     </row>
+    <row r="481" spans="1:12" ht="72" customHeight="1">
+      <c r="A481" s="4" t="s">
+        <v>2196</v>
+      </c>
+      <c r="B481" s="4" t="s">
+        <v>2197</v>
+      </c>
+      <c r="C481" s="4" t="s">
+        <v>2198</v>
+      </c>
+      <c r="D481" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E481" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F481" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G481" s="4" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H481" s="4" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I481" s="4" t="s">
+        <v>2201</v>
+      </c>
+      <c r="J481" s="4" t="s">
+        <v>2202</v>
+      </c>
+      <c r="K481" s="4" t="s">
+        <v>2203</v>
+      </c>
+      <c r="L481" s="6" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="482" spans="1:12" ht="72" customHeight="1">
+      <c r="A482" s="4" t="s">
+        <v>2204</v>
+      </c>
+      <c r="B482" s="4" t="s">
+        <v>2197</v>
+      </c>
+      <c r="C482" s="4" t="s">
+        <v>2205</v>
+      </c>
+      <c r="D482" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E482" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F482" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G482" s="4" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H482" s="4" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I482" s="4" t="s">
+        <v>2201</v>
+      </c>
+      <c r="J482" s="4" t="s">
+        <v>2206</v>
+      </c>
+      <c r="K482" s="4" t="s">
+        <v>2207</v>
+      </c>
+      <c r="L482" s="6" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="483" spans="1:12" ht="72" customHeight="1">
+      <c r="A483" s="4" t="s">
+        <v>2208</v>
+      </c>
+      <c r="B483" s="4" t="s">
+        <v>2197</v>
+      </c>
+      <c r="C483" s="4" t="s">
+        <v>2209</v>
+      </c>
+      <c r="D483" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E483" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F483" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G483" s="4" t="s">
+        <v>2199</v>
+      </c>
+      <c r="H483" s="4" t="s">
+        <v>2200</v>
+      </c>
+      <c r="I483" s="4" t="s">
+        <v>2201</v>
+      </c>
+      <c r="J483" s="4" t="s">
+        <v>2210</v>
+      </c>
+      <c r="K483" s="4" t="s">
+        <v>2211</v>
+      </c>
+      <c r="L483" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F480">
+  <conditionalFormatting sqref="E2:F483">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -46686,11 +46836,14 @@
     <hyperlink ref="L478" r:id="rId477"/>
     <hyperlink ref="L479" r:id="rId478"/>
     <hyperlink ref="L480" r:id="rId479"/>
+    <hyperlink ref="L481" r:id="rId480"/>
+    <hyperlink ref="L482" r:id="rId481"/>
+    <hyperlink ref="L483" r:id="rId482"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId480"/>
+    <tablePart r:id="rId483"/>
   </tableParts>
 </worksheet>
 </file>
@@ -46707,3128 +46860,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2446</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2447</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2295</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2448</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2263</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2442</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2443</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2444</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2292</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2445</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2260</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2439</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2440</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2593</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2295</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2594</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2263</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2590</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2292</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2591</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2260</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2587</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2641</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2642</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2320</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2643</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2637</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2644</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2638</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2639</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2317</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2640</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2634</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2641</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2635</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2650</v>
+        <v>2653</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
+        <v>2683</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2236</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>2684</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>2237</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>2680</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>2233</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
+        <v>2235</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>2263</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>2681</v>
       </c>
-      <c r="D95" s="4" t="s">
-        <v>2234</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>2677</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>2232</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>2260</v>
-      </c>
-      <c r="H95" s="4" t="s">
-        <v>2678</v>
-      </c>
       <c r="I95" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2685</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2239</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2680</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2263</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2681</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2682</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2236</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2683</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2237</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2677</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2235</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2260</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2678</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2679</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recover implemented companion tasks from legacy desktop handoffs
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12669" uniqueCount="2693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12699" uniqueCount="2696">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 13:54 BST</t>
+    <t>Snapshot: 07 September 2026, 14:00 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6666,6 +6666,15 @@
   </si>
   <si>
     <t>Surface handoff and preserved destination</t>
+  </si>
+  <si>
+    <t>Legacy handoff promotes documented direct companion routes via normalized local destination +both actual proxy capability predicates; unsupported requests show full-width honest fallback and useful tasks. Unit3PASS covers external/internal loops/unknown descendants/repeated filters/hash. Browser all6 layout,exact full-sitehref,canonicalProgress redirect and query/hash assertions pass; overall browser test fails on Next Performance.measure negative timestamp. Types/lint pass.</t>
+  </si>
+  <si>
+    <t>Full visible handoff at390/360/1023, large wrapped primary/alternative actions and exact requested context;390capture inspected. Promoted tasks go to canonical full mobile page. No handoff treated as completion of underlying blocked workflow.</t>
+  </si>
+  <si>
+    <t>handoff-browser-ready.log overall FAILED solely final pageerror assertion: Next CompanionHandoffPage Performance.measure negative time stamp recurred twice after successful navigation. Framework/runtime diagnosis deferred; no suppression applied. Full both-surface/role/entity/physicalkeyboard/AT/zoom/theme matrix outstanding; unsupported routes remain genuine fallback, not completed workflows.</t>
   </si>
   <si>
     <t>Switching surfaces preserves next, compareClub, compareMeasure and other valid query context without redirect loops.</t>
@@ -8272,8 +8281,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L483" totalsRowShown="0">
-  <autoFilter ref="A1:L483"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L485" totalsRowShown="0">
+  <autoFilter ref="A1:L485"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8667,11 +8676,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8706,11 +8715,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -27180,16 +27189,25 @@
         <v>32</v>
       </c>
       <c r="E484" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F484" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G484" s="4" t="s">
+        <v>2215</v>
+      </c>
+      <c r="H484" s="4" t="s">
+        <v>2216</v>
+      </c>
+      <c r="I484" s="4" t="s">
+        <v>2217</v>
       </c>
       <c r="J484" s="4" t="s">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="K484" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="L484" s="6" t="s">
         <v>165</v>
@@ -27197,28 +27215,37 @@
     </row>
     <row r="485" spans="1:12" ht="72" customHeight="1">
       <c r="A485" s="4" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="B485" s="4" t="s">
         <v>2213</v>
       </c>
       <c r="C485" s="4" t="s">
-        <v>2218</v>
+        <v>2221</v>
       </c>
       <c r="D485" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E485" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F485" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G485" s="4" t="s">
+        <v>2215</v>
+      </c>
+      <c r="H485" s="4" t="s">
+        <v>2216</v>
+      </c>
+      <c r="I485" s="4" t="s">
+        <v>2217</v>
       </c>
       <c r="J485" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="K485" s="4" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="L485" s="6" t="s">
         <v>110</v>
@@ -27226,13 +27253,13 @@
     </row>
     <row r="486" spans="1:12" ht="72" customHeight="1">
       <c r="A486" s="4" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="B486" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="C486" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D486" s="4" t="s">
         <v>42</v>
@@ -27244,10 +27271,10 @@
         <v>9</v>
       </c>
       <c r="J486" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="K486" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="L486" s="6" t="s">
         <v>165</v>
@@ -27255,13 +27282,13 @@
     </row>
     <row r="487" spans="1:12" ht="72" customHeight="1">
       <c r="A487" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="B487" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="C487" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="D487" s="4" t="s">
         <v>42</v>
@@ -27273,10 +27300,10 @@
         <v>9</v>
       </c>
       <c r="J487" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="K487" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="L487" s="6" t="s">
         <v>165</v>
@@ -27284,13 +27311,13 @@
     </row>
     <row r="488" spans="1:12" ht="72" customHeight="1">
       <c r="A488" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="B488" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="C488" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="D488" s="4" t="s">
         <v>42</v>
@@ -27302,10 +27329,10 @@
         <v>9</v>
       </c>
       <c r="J488" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="K488" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="L488" s="6" t="s">
         <v>141</v>
@@ -27313,13 +27340,13 @@
     </row>
     <row r="489" spans="1:12" ht="72" customHeight="1">
       <c r="A489" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="B489" s="4" t="s">
+        <v>2239</v>
+      </c>
+      <c r="C489" s="4" t="s">
         <v>2235</v>
-      </c>
-      <c r="B489" s="4" t="s">
-        <v>2236</v>
-      </c>
-      <c r="C489" s="4" t="s">
-        <v>2232</v>
       </c>
       <c r="D489" s="4" t="s">
         <v>42</v>
@@ -27331,10 +27358,10 @@
         <v>9</v>
       </c>
       <c r="J489" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27342,13 +27369,13 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C490" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="D490" s="4" t="s">
         <v>42</v>
@@ -27360,10 +27387,10 @@
         <v>9</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27371,13 +27398,13 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C491" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="D491" s="4" t="s">
         <v>42</v>
@@ -27389,10 +27416,10 @@
         <v>9</v>
       </c>
       <c r="J491" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27400,13 +27427,13 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C492" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="D492" s="4" t="s">
         <v>42</v>
@@ -27418,10 +27445,10 @@
         <v>9</v>
       </c>
       <c r="J492" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27429,13 +27456,13 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C493" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="D493" s="4" t="s">
         <v>42</v>
@@ -27447,10 +27474,10 @@
         <v>9</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -27981,7 +28008,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L483"/>
+  <dimension ref="A1:L485"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46338,8 +46365,84 @@
         <v>110</v>
       </c>
     </row>
+    <row r="484" spans="1:12" ht="72" customHeight="1">
+      <c r="A484" s="4" t="s">
+        <v>2212</v>
+      </c>
+      <c r="B484" s="4" t="s">
+        <v>2213</v>
+      </c>
+      <c r="C484" s="4" t="s">
+        <v>2214</v>
+      </c>
+      <c r="D484" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E484" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F484" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G484" s="4" t="s">
+        <v>2215</v>
+      </c>
+      <c r="H484" s="4" t="s">
+        <v>2216</v>
+      </c>
+      <c r="I484" s="4" t="s">
+        <v>2217</v>
+      </c>
+      <c r="J484" s="4" t="s">
+        <v>2218</v>
+      </c>
+      <c r="K484" s="4" t="s">
+        <v>2219</v>
+      </c>
+      <c r="L484" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="485" spans="1:12" ht="72" customHeight="1">
+      <c r="A485" s="4" t="s">
+        <v>2220</v>
+      </c>
+      <c r="B485" s="4" t="s">
+        <v>2213</v>
+      </c>
+      <c r="C485" s="4" t="s">
+        <v>2221</v>
+      </c>
+      <c r="D485" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E485" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F485" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G485" s="4" t="s">
+        <v>2215</v>
+      </c>
+      <c r="H485" s="4" t="s">
+        <v>2216</v>
+      </c>
+      <c r="I485" s="4" t="s">
+        <v>2217</v>
+      </c>
+      <c r="J485" s="4" t="s">
+        <v>2222</v>
+      </c>
+      <c r="K485" s="4" t="s">
+        <v>2223</v>
+      </c>
+      <c r="L485" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F483">
+  <conditionalFormatting sqref="E2:F485">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -46839,11 +46942,13 @@
     <hyperlink ref="L481" r:id="rId480"/>
     <hyperlink ref="L482" r:id="rId481"/>
     <hyperlink ref="L483" r:id="rId482"/>
+    <hyperlink ref="L484" r:id="rId483"/>
+    <hyperlink ref="L485" r:id="rId484"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId483"/>
+    <tablePart r:id="rId485"/>
   </tableParts>
 </worksheet>
 </file>
@@ -46860,3128 +46965,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2449</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2450</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2298</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2451</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2266</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2445</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2446</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2447</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2295</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2448</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2263</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2442</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2443</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2298</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2266</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2593</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2295</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2594</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2263</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2590</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2644</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2645</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2323</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2646</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2640</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2647</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2641</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2642</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2320</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2643</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2637</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2644</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2638</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2650</v>
+        <v>2653</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>2207</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>2213</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2239</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>2687</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>2683</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>2236</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>2266</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>2684</v>
       </c>
-      <c r="D95" s="4" t="s">
-        <v>2237</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>2680</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>2235</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>2263</v>
-      </c>
-      <c r="H95" s="4" t="s">
-        <v>2681</v>
-      </c>
       <c r="I95" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2688</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2689</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2243</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2683</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2241</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2266</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2684</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2685</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2239</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2686</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2240</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2680</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2238</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2263</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2681</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2682</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2692</v>
+        <v>2695</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace obsolete summaries with direct tasks and contextual fallbacks
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12699" uniqueCount="2696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12729" uniqueCount="2699">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 14:00 BST</t>
+    <t>Snapshot: 07 September 2026, 14:02 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6702,6 +6702,15 @@
   </si>
   <si>
     <t>Route-specific summary and next action</t>
+  </si>
+  <si>
+    <t>Known promoted routes use shared safe canonical redirect; remaining summaries now full-width with single heading/action, exact requested query context, semantic current evidence and explicit deeper-workflow limitation. Driver detail only for requested driver context. summary-browser.log1PASS20.8s all12surface/viewports empty summary, retained full-workspacehref, no unrelated driver/nooverflow/errors; types/lint clean.</t>
+  </si>
+  <si>
+    <t>Same full summary rows/context/primary/return actions at390/360/1023 on both surfaces;390 screenshot inspected. Actual implemented routes bypass legacy summary; fallback does not claim underlying mobile task completion.</t>
+  </si>
+  <si>
+    <t>Populated summaries/driver disclosure/native keyboard/AT/zoom/theme/service-error combinations outstanding. Shared redirect helper3unitPASS; P91 Next redirect Performance.measure defect may affect promoted summary redirects and is not resolved here. No fallback used to mark deeper workflow fully accepted.</t>
   </si>
   <si>
     <t>Summary content and destination correspond to the original requested route and selected entity.</t>
@@ -8281,8 +8290,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L485" totalsRowShown="0">
-  <autoFilter ref="A1:L485"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L487" totalsRowShown="0">
+  <autoFilter ref="A1:L487"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8676,11 +8685,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8715,11 +8724,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -27265,16 +27274,25 @@
         <v>42</v>
       </c>
       <c r="E486" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F486" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G486" s="4" t="s">
+        <v>2227</v>
+      </c>
+      <c r="H486" s="4" t="s">
+        <v>2228</v>
+      </c>
+      <c r="I486" s="4" t="s">
+        <v>2229</v>
       </c>
       <c r="J486" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="K486" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="L486" s="6" t="s">
         <v>165</v>
@@ -27282,28 +27300,37 @@
     </row>
     <row r="487" spans="1:12" ht="72" customHeight="1">
       <c r="A487" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="B487" s="4" t="s">
         <v>2225</v>
       </c>
       <c r="C487" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="D487" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E487" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F487" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G487" s="4" t="s">
+        <v>2227</v>
+      </c>
+      <c r="H487" s="4" t="s">
+        <v>2228</v>
+      </c>
+      <c r="I487" s="4" t="s">
+        <v>2229</v>
       </c>
       <c r="J487" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="K487" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="L487" s="6" t="s">
         <v>165</v>
@@ -27311,13 +27338,13 @@
     </row>
     <row r="488" spans="1:12" ht="72" customHeight="1">
       <c r="A488" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="B488" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="C488" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="D488" s="4" t="s">
         <v>42</v>
@@ -27329,10 +27356,10 @@
         <v>9</v>
       </c>
       <c r="J488" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="K488" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="L488" s="6" t="s">
         <v>141</v>
@@ -27340,13 +27367,13 @@
     </row>
     <row r="489" spans="1:12" ht="72" customHeight="1">
       <c r="A489" s="4" t="s">
+        <v>2241</v>
+      </c>
+      <c r="B489" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C489" s="4" t="s">
         <v>2238</v>
-      </c>
-      <c r="B489" s="4" t="s">
-        <v>2239</v>
-      </c>
-      <c r="C489" s="4" t="s">
-        <v>2235</v>
       </c>
       <c r="D489" s="4" t="s">
         <v>42</v>
@@ -27358,10 +27385,10 @@
         <v>9</v>
       </c>
       <c r="J489" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27369,13 +27396,13 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C490" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="D490" s="4" t="s">
         <v>42</v>
@@ -27387,10 +27414,10 @@
         <v>9</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27398,13 +27425,13 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C491" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="D491" s="4" t="s">
         <v>42</v>
@@ -27416,10 +27443,10 @@
         <v>9</v>
       </c>
       <c r="J491" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27427,13 +27454,13 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C492" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="D492" s="4" t="s">
         <v>42</v>
@@ -27445,10 +27472,10 @@
         <v>9</v>
       </c>
       <c r="J492" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27456,13 +27483,13 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="C493" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="D493" s="4" t="s">
         <v>42</v>
@@ -27474,10 +27501,10 @@
         <v>9</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -28008,7 +28035,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L487"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46441,8 +46468,84 @@
         <v>110</v>
       </c>
     </row>
+    <row r="486" spans="1:12" ht="72" customHeight="1">
+      <c r="A486" s="4" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B486" s="4" t="s">
+        <v>2225</v>
+      </c>
+      <c r="C486" s="4" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D486" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E486" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F486" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G486" s="4" t="s">
+        <v>2227</v>
+      </c>
+      <c r="H486" s="4" t="s">
+        <v>2228</v>
+      </c>
+      <c r="I486" s="4" t="s">
+        <v>2229</v>
+      </c>
+      <c r="J486" s="4" t="s">
+        <v>2230</v>
+      </c>
+      <c r="K486" s="4" t="s">
+        <v>2231</v>
+      </c>
+      <c r="L486" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="487" spans="1:12" ht="72" customHeight="1">
+      <c r="A487" s="4" t="s">
+        <v>2232</v>
+      </c>
+      <c r="B487" s="4" t="s">
+        <v>2225</v>
+      </c>
+      <c r="C487" s="4" t="s">
+        <v>2233</v>
+      </c>
+      <c r="D487" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E487" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F487" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G487" s="4" t="s">
+        <v>2227</v>
+      </c>
+      <c r="H487" s="4" t="s">
+        <v>2228</v>
+      </c>
+      <c r="I487" s="4" t="s">
+        <v>2229</v>
+      </c>
+      <c r="J487" s="4" t="s">
+        <v>2234</v>
+      </c>
+      <c r="K487" s="4" t="s">
+        <v>2235</v>
+      </c>
+      <c r="L487" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F485">
+  <conditionalFormatting sqref="E2:F487">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -46944,11 +47047,13 @@
     <hyperlink ref="L483" r:id="rId482"/>
     <hyperlink ref="L484" r:id="rId483"/>
     <hyperlink ref="L485" r:id="rId484"/>
+    <hyperlink ref="L486" r:id="rId485"/>
+    <hyperlink ref="L487" r:id="rId486"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId485"/>
+    <tablePart r:id="rId487"/>
   </tableParts>
 </worksheet>
 </file>
@@ -46965,3128 +47070,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2452</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2453</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2301</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2454</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2269</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2448</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2449</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2450</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2298</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2451</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2266</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2445</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2446</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2599</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2301</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2600</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2269</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2596</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2298</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2597</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2266</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2593</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2647</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2648</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2326</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2649</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2643</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2650</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2644</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2645</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2323</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2646</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2640</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2647</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2641</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2650</v>
+        <v>2653</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>2207</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>2213</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>2223</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>2225</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
+        <v>2689</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>2690</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>2243</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>2686</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>2239</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
+        <v>2241</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>2269</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>2687</v>
       </c>
-      <c r="D95" s="4" t="s">
-        <v>2240</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>2683</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>2238</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>2266</v>
-      </c>
-      <c r="H95" s="4" t="s">
-        <v>2684</v>
-      </c>
       <c r="I95" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2691</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2245</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2692</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2246</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2244</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2269</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2687</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2688</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2242</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2689</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2243</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2683</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2241</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2266</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2684</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2685</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2692</v>
+        <v>2695</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2693</v>
+        <v>2696</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2694</v>
+        <v>2697</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2695</v>
+        <v>2698</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore summary primary action styling and touch target
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 14:02 BST</t>
+    <t>Snapshot: 07 September 2026, 14:05 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6704,10 +6704,10 @@
     <t>Route-specific summary and next action</t>
   </si>
   <si>
-    <t>Known promoted routes use shared safe canonical redirect; remaining summaries now full-width with single heading/action, exact requested query context, semantic current evidence and explicit deeper-workflow limitation. Driver detail only for requested driver context. summary-browser.log1PASS20.8s all12surface/viewports empty summary, retained full-workspacehref, no unrelated driver/nooverflow/errors; types/lint clean.</t>
-  </si>
-  <si>
-    <t>Same full summary rows/context/primary/return actions at390/360/1023 on both surfaces;390 screenshot inspected. Actual implemented routes bypass legacy summary; fallback does not claim underlying mobile task completion.</t>
+    <t>Known promoted routes use shared safe canonical redirect; remaining summaries now full-width with single heading/action, exact requested query context, semantic current evidence and explicit deeper-workflow limitation. Driver detail only for requested driver context. summary-browser.log1PASS20.8s all12surface/viewports empty summary, retained full-workspacehref, no unrelated driver/nooverflow/errors; types/lint clean. Screenshot regression fixed: primary Link now receives Button props directly. summary-browser-final.log1PASS11.9s all12 and44pxprimarytarget.</t>
+  </si>
+  <si>
+    <t>Same full summary rows/context/primary/return actions at390/360/1023 on both surfaces;390 screenshot inspected. Actual implemented routes bypass legacy summary; fallback does not claim underlying mobile task completion. Same final11.9s run verifies primary link44px after wrapper styling regression fixed.</t>
   </si>
   <si>
     <t>Populated summaries/driver disclosure/native keyboard/AT/zoom/theme/service-error combinations outstanding. Shared redirect helper3unitPASS; P91 Next redirect Performance.measure defect may affect promoted summary redirects and is not resolved here. No fallback used to mark deeper workflow fully accepted.</t>

</xml_diff>

<commit_message>
Preserve record identity and query through canonical course aliases
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12729" uniqueCount="2699">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12744" uniqueCount="2702">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 14:05 BST</t>
+    <t>Snapshot: 07 September 2026, 14:08 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6738,6 +6738,15 @@
   </si>
   <si>
     <t>Canonical destination and selected component</t>
+  </si>
+  <si>
+    <t>Server alias encodes exact recordId and retains repeated query values. Companion proxy now permits alias to canonical record task. record-alias-browser.log1PASS53.3s all12surface/viewports exactnamedrecord/form/query, nooverflow/errors and no additional attempts;390reload/Back return exactcanonicalURL. Query helper2unitPASS; types clean.</t>
+  </si>
+  <si>
+    <t>Same canonical P57 full record task reached on390/360/1023 both surfaces; P93 captures. Course segment remains alias, not separate editor; receipt/filter query retained.</t>
+  </si>
+  <si>
+    <t>Invalid/foreign record alias browser cases, Forward, native keyboard/AT/zoom/theme matrices outstanding. Destination P57 full acceptance stillpartial. Canonicalalias adds no separate Untitled tabs or duplicate editor.</t>
   </si>
   <si>
     <t>Direct navigation, reload and Back/Forward reach the correct canonical task; invalid IDs still respect access/not-found handling.</t>
@@ -8290,8 +8299,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L487" totalsRowShown="0">
-  <autoFilter ref="A1:L487"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L488" totalsRowShown="0">
+  <autoFilter ref="A1:L488"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8685,11 +8694,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8724,11 +8733,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -27350,16 +27359,25 @@
         <v>42</v>
       </c>
       <c r="E488" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F488" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G488" s="4" t="s">
+        <v>2239</v>
+      </c>
+      <c r="H488" s="4" t="s">
+        <v>2240</v>
+      </c>
+      <c r="I488" s="4" t="s">
+        <v>2241</v>
       </c>
       <c r="J488" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="K488" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="L488" s="6" t="s">
         <v>141</v>
@@ -27367,10 +27385,10 @@
     </row>
     <row r="489" spans="1:12" ht="72" customHeight="1">
       <c r="A489" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="B489" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="C489" s="4" t="s">
         <v>2238</v>
@@ -27385,10 +27403,10 @@
         <v>9</v>
       </c>
       <c r="J489" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27396,10 +27414,10 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="C490" s="4" t="s">
         <v>2238</v>
@@ -27414,10 +27432,10 @@
         <v>9</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27425,10 +27443,10 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C491" s="4" t="s">
         <v>2238</v>
@@ -27443,10 +27461,10 @@
         <v>9</v>
       </c>
       <c r="J491" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27454,10 +27472,10 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="C492" s="4" t="s">
         <v>2238</v>
@@ -27472,10 +27490,10 @@
         <v>9</v>
       </c>
       <c r="J492" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27483,10 +27501,10 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="C493" s="4" t="s">
         <v>2238</v>
@@ -27501,10 +27519,10 @@
         <v>9</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -28035,7 +28053,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L487"/>
+  <dimension ref="A1:L488"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46544,8 +46562,46 @@
         <v>165</v>
       </c>
     </row>
+    <row r="488" spans="1:12" ht="72" customHeight="1">
+      <c r="A488" s="4" t="s">
+        <v>2236</v>
+      </c>
+      <c r="B488" s="4" t="s">
+        <v>2237</v>
+      </c>
+      <c r="C488" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D488" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E488" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F488" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G488" s="4" t="s">
+        <v>2239</v>
+      </c>
+      <c r="H488" s="4" t="s">
+        <v>2240</v>
+      </c>
+      <c r="I488" s="4" t="s">
+        <v>2241</v>
+      </c>
+      <c r="J488" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="K488" s="4" t="s">
+        <v>2243</v>
+      </c>
+      <c r="L488" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F487">
+  <conditionalFormatting sqref="E2:F488">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -47049,11 +47105,12 @@
     <hyperlink ref="L485" r:id="rId484"/>
     <hyperlink ref="L486" r:id="rId485"/>
     <hyperlink ref="L487" r:id="rId486"/>
+    <hyperlink ref="L488" r:id="rId487"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId487"/>
+    <tablePart r:id="rId488"/>
   </tableParts>
 </worksheet>
 </file>
@@ -47070,3128 +47127,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2455</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2456</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2304</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2457</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2272</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2451</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2452</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2453</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2301</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2454</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2269</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2448</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2449</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2602</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2304</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2603</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2272</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2599</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2301</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2600</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2269</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2596</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2650</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2651</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2329</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2652</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2646</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2653</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2647</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2648</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2326</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2649</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2643</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2650</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2644</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>2207</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>2213</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>2223</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>2225</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>2231</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>2237</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>2236</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
+        <v>2692</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2245</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>2693</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>2246</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>2689</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>2242</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
+        <v>2244</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>2272</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>2690</v>
       </c>
-      <c r="D95" s="4" t="s">
-        <v>2243</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>2686</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>2241</v>
-      </c>
-      <c r="G95" s="4" t="s">
-        <v>2269</v>
-      </c>
-      <c r="H95" s="4" t="s">
-        <v>2687</v>
-      </c>
       <c r="I95" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2694</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2248</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2695</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2249</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2689</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2247</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2272</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2690</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2691</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2245</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2692</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2246</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2686</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2244</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2269</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2687</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2688</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2693</v>
+        <v>2696</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2694</v>
+        <v>2697</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2695</v>
+        <v>2698</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2696</v>
+        <v>2699</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2697</v>
+        <v>2700</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2698</v>
+        <v>2701</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Retain tournament filters through canonical course navigation
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12744" uniqueCount="2702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12759" uniqueCount="2705">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 14:08 BST</t>
+    <t>Snapshot: 07 September 2026, 14:12 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6759,6 +6759,15 @@
   </si>
   <si>
     <t>/courses/[courseId]/tournaments</t>
+  </si>
+  <si>
+    <t>Server alias retains query and forces path courseId over conflicting supplied query. course-tournament-alias-browser-final.log all12surface/viewports exactURL/coursefilter/activepanel/matching event only/nooverflow assertions pass; overall testFAIL Next Performance.measure negative timestamp finalpageerror. Queryhelper3unitPASS/typesclean.</t>
+  </si>
+  <si>
+    <t>390/360/1023 bothsurfaces open full P60 tournament task with same visible selectedcourse and matchingevents, no other venue event. P94 captures; destination full UI retained.</t>
+  </si>
+  <si>
+    <t>Overall browser test fails development-runtime CourseTournamentsPage negative timestamp; no suppression. Earlier fixture assertion chose hidden desktop copy onphone, corrected visible presentation. Reload/Back/Forward/invalidcourse/nativeAT/zoom/themes remain outstanding; P60 acceptance stillpartial.</t>
   </si>
   <si>
     <t>src/app/(app)/courses/[courseId]/tournaments/page.tsx</t>
@@ -8299,8 +8308,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L488" totalsRowShown="0">
-  <autoFilter ref="A1:L488"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L489" totalsRowShown="0">
+  <autoFilter ref="A1:L489"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8694,11 +8703,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8733,11 +8742,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -27397,16 +27406,25 @@
         <v>42</v>
       </c>
       <c r="E489" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F489" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G489" s="4" t="s">
+        <v>2246</v>
+      </c>
+      <c r="H489" s="4" t="s">
+        <v>2247</v>
+      </c>
+      <c r="I489" s="4" t="s">
+        <v>2248</v>
       </c>
       <c r="J489" s="4" t="s">
         <v>2242</v>
       </c>
       <c r="K489" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="L489" s="6" t="s">
         <v>141</v>
@@ -27414,10 +27432,10 @@
     </row>
     <row r="490" spans="1:12" ht="72" customHeight="1">
       <c r="A490" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="C490" s="4" t="s">
         <v>2238</v>
@@ -27435,7 +27453,7 @@
         <v>2242</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27443,10 +27461,10 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="C491" s="4" t="s">
         <v>2238</v>
@@ -27464,7 +27482,7 @@
         <v>2242</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27472,10 +27490,10 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="C492" s="4" t="s">
         <v>2238</v>
@@ -27493,7 +27511,7 @@
         <v>2242</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27501,10 +27519,10 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="C493" s="4" t="s">
         <v>2238</v>
@@ -27522,7 +27540,7 @@
         <v>2242</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -28053,7 +28071,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L488"/>
+  <dimension ref="A1:L489"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46600,8 +46618,46 @@
         <v>141</v>
       </c>
     </row>
+    <row r="489" spans="1:12" ht="72" customHeight="1">
+      <c r="A489" s="4" t="s">
+        <v>2244</v>
+      </c>
+      <c r="B489" s="4" t="s">
+        <v>2245</v>
+      </c>
+      <c r="C489" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D489" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E489" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F489" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G489" s="4" t="s">
+        <v>2246</v>
+      </c>
+      <c r="H489" s="4" t="s">
+        <v>2247</v>
+      </c>
+      <c r="I489" s="4" t="s">
+        <v>2248</v>
+      </c>
+      <c r="J489" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="K489" s="4" t="s">
+        <v>2249</v>
+      </c>
+      <c r="L489" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F488">
+  <conditionalFormatting sqref="E2:F489">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -47106,11 +47162,12 @@
     <hyperlink ref="L486" r:id="rId485"/>
     <hyperlink ref="L487" r:id="rId486"/>
     <hyperlink ref="L488" r:id="rId487"/>
+    <hyperlink ref="L489" r:id="rId488"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId488"/>
+    <tablePart r:id="rId489"/>
   </tableParts>
 </worksheet>
 </file>
@@ -47127,3128 +47184,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>2458</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>2459</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>2307</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>2460</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>2454</v>
+      </c>
+      <c r="I41" s="4" t="s">
         <v>2455</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>2456</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>2304</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>2457</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>2272</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>2451</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>2452</v>
-      </c>
       <c r="J41" s="4" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="D75" s="4" t="s">
+        <v>2605</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2307</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2606</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2602</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>2304</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2603</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2272</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2599</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
+        <v>2653</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>2654</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>2332</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>2655</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>2649</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>2656</v>
+      </c>
+      <c r="I85" s="4" t="s">
         <v>2650</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>2651</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>2329</v>
-      </c>
-      <c r="F85" s="4" t="s">
-        <v>2652</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>2646</v>
-      </c>
-      <c r="H85" s="4" t="s">
-        <v>2653</v>
-      </c>
-      <c r="I85" s="4" t="s">
-        <v>2647</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>2207</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>2213</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>2223</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>2225</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2685</v>
+        <v>2688</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>2231</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2686</v>
+        <v>2689</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2687</v>
+        <v>2690</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>2237</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2688</v>
+        <v>2691</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>2243</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>2236</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
-        <v>2692</v>
+        <v>2695</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>2245</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>2693</v>
+        <v>2696</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>2244</v>
       </c>
       <c r="G95" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H95" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
+        <v>2697</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>2251</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2698</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>2692</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>2250</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>2275</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>2693</v>
+      </c>
+      <c r="I96" s="4" t="s">
         <v>2694</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>2248</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>2695</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>2249</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>2689</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>2247</v>
-      </c>
-      <c r="G96" s="4" t="s">
-        <v>2272</v>
-      </c>
-      <c r="H96" s="4" t="s">
-        <v>2690</v>
-      </c>
-      <c r="I96" s="4" t="s">
-        <v>2691</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2696</v>
+        <v>2699</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2697</v>
+        <v>2700</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2698</v>
+        <v>2701</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2699</v>
+        <v>2702</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2700</v>
+        <v>2703</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2701</v>
+        <v>2704</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>2689</v>
+        <v>2692</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2690</v>
+        <v>2693</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2691</v>
+        <v>2694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Preserve tournament alias context across canonical panels
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12759" uniqueCount="2705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12819" uniqueCount="2707">
   <si>
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 14:12 BST</t>
+    <t>Snapshot: 07 September 2026, 14:42 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6777,6 +6777,12 @@
   </si>
   <si>
     <t>/tournaments/[tournamentId]/leaderboard</t>
+  </si>
+  <si>
+    <t>Both explicit surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800 reached exact event/panel, preserved repeated query filters, no horizontal overflow; 390 reload/Back retained URL; zero fixture entry mutations. All four tests failed their final page-error assertion with Next development Performance.measure negative timestamp errors. Log tournament-alias-browser.log. Seven canonical-query unit tests pass; scoped types/lint clean.</t>
+  </si>
+  <si>
+    <t>Browser suite not passing: development Performance.measure negative timestamp for redirect component. Capture stack and compare isolated production runtime; do not suppress. Invalid/foreign event, Forward, native browser, screen reader, themes and full acceptance outstanding.</t>
   </si>
   <si>
     <t>src/app/(app)/tournaments/[tournamentId]/leaderboard/page.tsx</t>
@@ -8308,8 +8314,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L489" totalsRowShown="0">
-  <autoFilter ref="A1:L489"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:L493" totalsRowShown="0">
+  <autoFilter ref="A1:L493"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Component ID"/>
     <tableColumn id="2" name="Route"/>
@@ -8703,11 +8709,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Components!E2:E493,"Implemented; partial verification")</f>
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Components!F2:F493,"Implemented; partial verification")</f>
-        <v>481</v>
+        <v>485</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8742,11 +8748,11 @@
       </c>
       <c r="B13" s="5">
         <f>COUNTIF(Components!E2:E493,"Not started")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C13" s="5">
         <f>COUNTIF(Components!F2:F493,"Not started")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -27444,16 +27450,25 @@
         <v>42</v>
       </c>
       <c r="E490" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F490" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G490" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H490" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I490" s="4" t="s">
+        <v>2253</v>
       </c>
       <c r="J490" s="4" t="s">
         <v>2242</v>
       </c>
       <c r="K490" s="4" t="s">
-        <v>2252</v>
+        <v>2254</v>
       </c>
       <c r="L490" s="6" t="s">
         <v>141</v>
@@ -27461,10 +27476,10 @@
     </row>
     <row r="491" spans="1:12" ht="72" customHeight="1">
       <c r="A491" s="4" t="s">
-        <v>2253</v>
+        <v>2255</v>
       </c>
       <c r="B491" s="4" t="s">
-        <v>2254</v>
+        <v>2256</v>
       </c>
       <c r="C491" s="4" t="s">
         <v>2238</v>
@@ -27473,16 +27488,25 @@
         <v>42</v>
       </c>
       <c r="E491" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F491" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G491" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H491" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I491" s="4" t="s">
+        <v>2253</v>
       </c>
       <c r="J491" s="4" t="s">
         <v>2242</v>
       </c>
       <c r="K491" s="4" t="s">
-        <v>2255</v>
+        <v>2257</v>
       </c>
       <c r="L491" s="6" t="s">
         <v>141</v>
@@ -27490,10 +27514,10 @@
     </row>
     <row r="492" spans="1:12" ht="72" customHeight="1">
       <c r="A492" s="4" t="s">
-        <v>2256</v>
+        <v>2258</v>
       </c>
       <c r="B492" s="4" t="s">
-        <v>2257</v>
+        <v>2259</v>
       </c>
       <c r="C492" s="4" t="s">
         <v>2238</v>
@@ -27502,16 +27526,25 @@
         <v>42</v>
       </c>
       <c r="E492" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F492" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G492" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H492" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I492" s="4" t="s">
+        <v>2253</v>
       </c>
       <c r="J492" s="4" t="s">
         <v>2242</v>
       </c>
       <c r="K492" s="4" t="s">
-        <v>2258</v>
+        <v>2260</v>
       </c>
       <c r="L492" s="6" t="s">
         <v>141</v>
@@ -27519,10 +27552,10 @@
     </row>
     <row r="493" spans="1:12" ht="72" customHeight="1">
       <c r="A493" s="4" t="s">
-        <v>2259</v>
+        <v>2261</v>
       </c>
       <c r="B493" s="4" t="s">
-        <v>2260</v>
+        <v>2262</v>
       </c>
       <c r="C493" s="4" t="s">
         <v>2238</v>
@@ -27531,16 +27564,25 @@
         <v>42</v>
       </c>
       <c r="E493" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F493" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="G493" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H493" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I493" s="4" t="s">
+        <v>2253</v>
       </c>
       <c r="J493" s="4" t="s">
         <v>2242</v>
       </c>
       <c r="K493" s="4" t="s">
-        <v>2261</v>
+        <v>2263</v>
       </c>
       <c r="L493" s="6" t="s">
         <v>141</v>
@@ -28071,7 +28113,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L489"/>
+  <dimension ref="A1:L493"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="4" customWidth="1"/>
@@ -46656,8 +46698,160 @@
         <v>141</v>
       </c>
     </row>
+    <row r="490" spans="1:12" ht="72" customHeight="1">
+      <c r="A490" s="4" t="s">
+        <v>2250</v>
+      </c>
+      <c r="B490" s="4" t="s">
+        <v>2251</v>
+      </c>
+      <c r="C490" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D490" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E490" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F490" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G490" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H490" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I490" s="4" t="s">
+        <v>2253</v>
+      </c>
+      <c r="J490" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="K490" s="4" t="s">
+        <v>2254</v>
+      </c>
+      <c r="L490" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="491" spans="1:12" ht="72" customHeight="1">
+      <c r="A491" s="4" t="s">
+        <v>2255</v>
+      </c>
+      <c r="B491" s="4" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C491" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D491" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E491" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F491" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G491" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H491" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I491" s="4" t="s">
+        <v>2253</v>
+      </c>
+      <c r="J491" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="K491" s="4" t="s">
+        <v>2257</v>
+      </c>
+      <c r="L491" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="492" spans="1:12" ht="72" customHeight="1">
+      <c r="A492" s="4" t="s">
+        <v>2258</v>
+      </c>
+      <c r="B492" s="4" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C492" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D492" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E492" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F492" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G492" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H492" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I492" s="4" t="s">
+        <v>2253</v>
+      </c>
+      <c r="J492" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="K492" s="4" t="s">
+        <v>2260</v>
+      </c>
+      <c r="L492" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="493" spans="1:12" ht="72" customHeight="1">
+      <c r="A493" s="4" t="s">
+        <v>2261</v>
+      </c>
+      <c r="B493" s="4" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C493" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D493" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E493" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F493" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G493" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="H493" s="4" t="s">
+        <v>2252</v>
+      </c>
+      <c r="I493" s="4" t="s">
+        <v>2253</v>
+      </c>
+      <c r="J493" s="4" t="s">
+        <v>2242</v>
+      </c>
+      <c r="K493" s="4" t="s">
+        <v>2263</v>
+      </c>
+      <c r="L493" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:F489">
+  <conditionalFormatting sqref="E2:F493">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Implemented; partial verification"</formula>
     </cfRule>
@@ -47163,11 +47357,15 @@
     <hyperlink ref="L487" r:id="rId486"/>
     <hyperlink ref="L488" r:id="rId487"/>
     <hyperlink ref="L489" r:id="rId488"/>
+    <hyperlink ref="L490" r:id="rId489"/>
+    <hyperlink ref="L491" r:id="rId490"/>
+    <hyperlink ref="L492" r:id="rId491"/>
+    <hyperlink ref="L493" r:id="rId492"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId489"/>
+    <tablePart r:id="rId493"/>
   </tableParts>
 </worksheet>
 </file>
@@ -47184,3128 +47382,3128 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>2262</v>
+        <v>2264</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2263</v>
+        <v>2265</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2264</v>
+        <v>2266</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>2265</v>
+        <v>2267</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2266</v>
+        <v>2268</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>2267</v>
+        <v>2269</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2268</v>
+        <v>2270</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2269</v>
+        <v>2271</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>2270</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="4" t="s">
-        <v>2271</v>
+        <v>2273</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2272</v>
+        <v>2274</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>134</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2273</v>
+        <v>2275</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>2274</v>
+        <v>2276</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>2278</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="4" t="s">
-        <v>2279</v>
+        <v>2281</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>2280</v>
+        <v>2282</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>230</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>2282</v>
+        <v>2284</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>2283</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="4" t="s">
-        <v>2284</v>
+        <v>2286</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>2285</v>
+        <v>2287</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>241</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2286</v>
+        <v>2288</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>2287</v>
+        <v>2289</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>2289</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="4" t="s">
-        <v>2290</v>
+        <v>2292</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>2291</v>
+        <v>2293</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2292</v>
+        <v>2294</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>2294</v>
+        <v>2296</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>2295</v>
+        <v>2297</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
-        <v>2296</v>
+        <v>2298</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>292</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>2297</v>
+        <v>2299</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>306</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>2286</v>
+        <v>2288</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>2298</v>
+        <v>2300</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>2299</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
-        <v>2300</v>
+        <v>2302</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>325</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>2301</v>
+        <v>2303</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>342</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>2302</v>
+        <v>2304</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>2303</v>
+        <v>2305</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
-        <v>2304</v>
+        <v>2306</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>347</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>2305</v>
+        <v>2307</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>2306</v>
+        <v>2308</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2308</v>
+        <v>2310</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>2309</v>
+        <v>2311</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
-        <v>2310</v>
+        <v>2312</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>2311</v>
+        <v>2313</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>368</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>2312</v>
+        <v>2314</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>2313</v>
+        <v>2315</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>2314</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="4" t="s">
-        <v>2315</v>
+        <v>2317</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>2316</v>
+        <v>2318</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>2317</v>
+        <v>2319</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>2319</v>
+        <v>2321</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>2320</v>
+        <v>2322</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="4" t="s">
-        <v>2321</v>
+        <v>2323</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>445</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>2322</v>
+        <v>2324</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>460</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>2323</v>
+        <v>2325</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>2324</v>
+        <v>2326</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="4" t="s">
-        <v>2325</v>
+        <v>2327</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>477</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2327</v>
+        <v>2329</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="4" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>490</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>2330</v>
+        <v>2332</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>2331</v>
+        <v>2333</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>2333</v>
+        <v>2335</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>2334</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="4" t="s">
-        <v>2335</v>
+        <v>2337</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>508</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>2336</v>
+        <v>2338</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>513</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2337</v>
+        <v>2339</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>2338</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="4" t="s">
-        <v>2339</v>
+        <v>2341</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>541</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>546</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>2341</v>
+        <v>2343</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>2342</v>
+        <v>2344</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="4" t="s">
-        <v>2343</v>
+        <v>2345</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>557</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>2344</v>
+        <v>2346</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>2345</v>
+        <v>2347</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>2346</v>
+        <v>2348</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>2347</v>
+        <v>2349</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="4" t="s">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>591</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2350</v>
+        <v>2352</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>2351</v>
+        <v>2353</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>2352</v>
+        <v>2354</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>2353</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="4" t="s">
-        <v>2354</v>
+        <v>2356</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>2355</v>
+        <v>2357</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>611</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>2356</v>
+        <v>2358</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="4" t="s">
-        <v>2359</v>
+        <v>2361</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>631</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>2360</v>
+        <v>2362</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>2361</v>
+        <v>2363</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>2362</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="4" t="s">
-        <v>2363</v>
+        <v>2365</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>646</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>2364</v>
+        <v>2366</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>656</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>2365</v>
+        <v>2367</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>2366</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="4" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>662</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>2368</v>
+        <v>2370</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>673</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>2369</v>
+        <v>2371</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>2370</v>
+        <v>2372</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="4" t="s">
-        <v>2371</v>
+        <v>2373</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>682</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>2372</v>
+        <v>2374</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>698</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>2373</v>
+        <v>2375</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>2374</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="4" t="s">
-        <v>2375</v>
+        <v>2377</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>700</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>2376</v>
+        <v>2378</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>706</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>2377</v>
+        <v>2379</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>2378</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="4" t="s">
-        <v>2379</v>
+        <v>2381</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>721</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>2380</v>
+        <v>2382</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>2381</v>
+        <v>2383</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>2382</v>
+        <v>2384</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>2383</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="4" t="s">
-        <v>2384</v>
+        <v>2386</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>745</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>2385</v>
+        <v>2387</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>2386</v>
+        <v>2388</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>2387</v>
+        <v>2389</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2388</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="4" t="s">
-        <v>2389</v>
+        <v>2391</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>764</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>2390</v>
+        <v>2392</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>2391</v>
+        <v>2393</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>2392</v>
+        <v>2394</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>2393</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="4" t="s">
-        <v>2394</v>
+        <v>2396</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>781</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>2395</v>
+        <v>2397</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>787</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>2397</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="4" t="s">
-        <v>2398</v>
+        <v>2400</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>798</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2399</v>
+        <v>2401</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>2400</v>
+        <v>2402</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>2401</v>
+        <v>2403</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>2402</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="4" t="s">
-        <v>2403</v>
+        <v>2405</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>2404</v>
+        <v>2406</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>831</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>2286</v>
+        <v>2288</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>2405</v>
+        <v>2407</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>2406</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="4" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>851</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>2408</v>
+        <v>2410</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>865</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>2409</v>
+        <v>2411</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>2410</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="4" t="s">
-        <v>2411</v>
+        <v>2413</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>887</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>2412</v>
+        <v>2414</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>904</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>2413</v>
+        <v>2415</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>2414</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="4" t="s">
-        <v>2415</v>
+        <v>2417</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>922</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2416</v>
+        <v>2418</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>935</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>2417</v>
+        <v>2419</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="4" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>948</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>2420</v>
+        <v>2422</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>965</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>2421</v>
+        <v>2423</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>2422</v>
+        <v>2424</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="4" t="s">
-        <v>2423</v>
+        <v>2425</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>975</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>981</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>2425</v>
+        <v>2427</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>2426</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>2427</v>
+        <v>2429</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>1003</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>1008</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>1024</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>2273</v>
+        <v>2275</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>2434</v>
+        <v>2436</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>2435</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>2436</v>
+        <v>2438</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>1076</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>2437</v>
+        <v>2439</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>1081</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>2439</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>2440</v>
+        <v>2442</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>1092</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>2441</v>
+        <v>2443</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>2442</v>
+        <v>2444</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>2443</v>
+        <v>2445</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>2444</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>1108</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="D39" s="4" t="s">
         <v>1121</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>2449</v>
+        <v>2451</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2450</v>
+        <v>2452</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>2456</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="4" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>1148</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>2463</v>
+        <v>2465</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>1153</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>2464</v>
+        <v>2466</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>2465</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="4" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>1159</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>2467</v>
+        <v>2469</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>2468</v>
+        <v>2470</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>2469</v>
+        <v>2471</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>2470</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="4" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>1173</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>2473</v>
+        <v>2475</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>2475</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="4" t="s">
-        <v>2476</v>
+        <v>2478</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>1191</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>2477</v>
+        <v>2479</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>2478</v>
+        <v>2480</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>2479</v>
+        <v>2481</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>2480</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="4" t="s">
-        <v>2481</v>
+        <v>2483</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>1205</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>2482</v>
+        <v>2484</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>1210</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>2484</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="4" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>1242</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2486</v>
+        <v>2488</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>2488</v>
+        <v>2490</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="4" t="s">
-        <v>2490</v>
+        <v>2492</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>1257</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>2491</v>
+        <v>2493</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>1267</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>2493</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>2494</v>
+        <v>2496</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>1277</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>2495</v>
+        <v>2497</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>1290</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>2496</v>
+        <v>2498</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>2497</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>2498</v>
+        <v>2500</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>1298</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>2499</v>
+        <v>2501</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>1316</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>2286</v>
+        <v>2288</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>2500</v>
+        <v>2502</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>2501</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>2502</v>
+        <v>2504</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>1328</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>2503</v>
+        <v>2505</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>1334</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>2504</v>
+        <v>2506</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>2505</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>2506</v>
+        <v>2508</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>1346</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>2507</v>
+        <v>2509</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>1359</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>2508</v>
+        <v>2510</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2509</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>2510</v>
+        <v>2512</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>1367</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>2511</v>
+        <v>2513</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>2512</v>
+        <v>2514</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>2513</v>
+        <v>2515</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>2514</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>2515</v>
+        <v>2517</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>1377</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>1390</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>2517</v>
+        <v>2519</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>2518</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>2519</v>
+        <v>2521</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>1398</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>2520</v>
+        <v>2522</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>2521</v>
+        <v>2523</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>2522</v>
+        <v>2524</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>2523</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>2524</v>
+        <v>2526</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>1417</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>2525</v>
+        <v>2527</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>1426</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>2526</v>
+        <v>2528</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>2527</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>2528</v>
+        <v>2530</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>1432</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>2529</v>
+        <v>2531</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>1437</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>2530</v>
+        <v>2532</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>2531</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>2532</v>
+        <v>2534</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>1446</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>2533</v>
+        <v>2535</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>1463</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>2534</v>
+        <v>2536</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>2535</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>2536</v>
+        <v>2538</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>1468</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>2537</v>
+        <v>2539</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>1473</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>2538</v>
+        <v>2540</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>2539</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="4" t="s">
-        <v>2540</v>
+        <v>2542</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>1490</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>2541</v>
+        <v>2543</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>1499</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>2286</v>
+        <v>2288</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>2542</v>
+        <v>2544</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>2543</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="4" t="s">
-        <v>2544</v>
+        <v>2546</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>1519</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="D61" s="4" t="s">
         <v>1524</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>2546</v>
+        <v>2548</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>2547</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="4" t="s">
-        <v>2548</v>
+        <v>2550</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>1532</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>2549</v>
+        <v>2551</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>1538</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>2346</v>
+        <v>2348</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>2550</v>
+        <v>2552</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="4" t="s">
-        <v>2552</v>
+        <v>2554</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>1566</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>2553</v>
+        <v>2555</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>1580</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>2554</v>
+        <v>2556</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>2555</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="4" t="s">
-        <v>2556</v>
+        <v>2558</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>1588</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>2557</v>
+        <v>2559</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>1613</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>2558</v>
+        <v>2560</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>2559</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="4" t="s">
-        <v>2560</v>
+        <v>2562</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>1615</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>2561</v>
+        <v>2563</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>1629</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>2562</v>
+        <v>2564</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>2563</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="4" t="s">
-        <v>2564</v>
+        <v>2566</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>1635</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>2565</v>
+        <v>2567</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>1645</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>2567</v>
+        <v>2569</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="4" t="s">
-        <v>2568</v>
+        <v>2570</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>1654</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>2569</v>
+        <v>2571</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>1664</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>2570</v>
+        <v>2572</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>2571</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="4" t="s">
-        <v>2572</v>
+        <v>2574</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>1680</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>1698</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>2574</v>
+        <v>2576</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>2575</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="4" t="s">
-        <v>2576</v>
+        <v>2578</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>1700</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>1706</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="4" t="s">
-        <v>2580</v>
+        <v>2582</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>1718</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>2581</v>
+        <v>2583</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>1724</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="4" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>1755</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>1765</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>2587</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="4" t="s">
-        <v>2588</v>
+        <v>2590</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>1774</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>2589</v>
+        <v>2591</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>1780</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>2590</v>
+        <v>2592</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>2591</v>
+        <v>2593</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>2592</v>
+        <v>2594</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="4" t="s">
-        <v>2593</v>
+        <v>2595</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>1827</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>2594</v>
+        <v>2596</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>2595</v>
+        <v>2597</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>2596</v>
+        <v>2598</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="4" t="s">
-        <v>2598</v>
+        <v>2600</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>1843</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>2599</v>
+        <v>2601</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>2600</v>
+        <v>2602</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>2601</v>
+        <v>2603</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" s="4" t="s">
-        <v>2603</v>
+        <v>2605</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>1854</v>
       </c>
       <c r="C75" s="4" t="s">
+        <v>2606</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>2607</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>2309</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>2608</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>2277</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>2604</v>
       </c>
-      <c r="D75" s="4" t="s">
-        <v>2605</v>
-      </c>
-      <c r="E75" s="4" t="s">
-        <v>2307</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>2606</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>2275</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>2602</v>
-      </c>
       <c r="I75" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" s="4" t="s">
-        <v>2607</v>
+        <v>2609</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>1869</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>2608</v>
+        <v>2610</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>1875</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>2609</v>
+        <v>2611</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>2610</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="4" t="s">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>1895</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>2612</v>
+        <v>2614</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>2614</v>
+        <v>2616</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>2615</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="4" t="s">
-        <v>2616</v>
+        <v>2618</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>1918</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>2618</v>
+        <v>2620</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>2619</v>
+        <v>2621</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="4" t="s">
-        <v>2621</v>
+        <v>2623</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>1938</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>2624</v>
+        <v>2626</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>2625</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="4" t="s">
-        <v>2626</v>
+        <v>2628</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>1961</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>2627</v>
+        <v>2629</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>2628</v>
+        <v>2630</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>2629</v>
+        <v>2631</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>2630</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="4" t="s">
-        <v>2631</v>
+        <v>2633</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>1981</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>2632</v>
+        <v>2634</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>2633</v>
+        <v>2635</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>2634</v>
+        <v>2636</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="4" t="s">
-        <v>2636</v>
+        <v>2638</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>2000</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>2637</v>
+        <v>2639</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>2006</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>2638</v>
+        <v>2640</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>2639</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="4" t="s">
-        <v>2640</v>
+        <v>2642</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>2019</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>2641</v>
+        <v>2643</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>2025</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>2642</v>
+        <v>2644</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>2643</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="4" t="s">
-        <v>2644</v>
+        <v>2646</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>2042</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>2645</v>
+        <v>2647</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>2647</v>
+        <v>2649</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>2648</v>
+        <v>2650</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2651</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="4" t="s">
-        <v>2652</v>
+        <v>2654</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>2094</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>2654</v>
+        <v>2656</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>2655</v>
+        <v>2657</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>2656</v>
+        <v>2658</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="4" t="s">
-        <v>2657</v>
+        <v>2659</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>2114</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>2658</v>
+        <v>2660</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>2659</v>
+        <v>2661</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>2660</v>
+        <v>2662</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>2661</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="4" t="s">
-        <v>2662</v>
+        <v>2664</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>2128</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>2663</v>
+        <v>2665</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>2664</v>
+        <v>2666</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>2665</v>
+        <v>2667</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>2666</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="4" t="s">
-        <v>2667</v>
+        <v>2669</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>2143</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>2668</v>
+        <v>2670</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>2669</v>
+        <v>2671</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>2670</v>
+        <v>2672</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>2671</v>
+        <v>2673</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>2672</v>
+        <v>2674</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="A89" s="4" t="s">
-        <v>2673</v>
+        <v>2675</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>2167</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>2674</v>
+        <v>2676</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>2675</v>
+        <v>2677</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>2676</v>
+        <v>2678</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="4" t="s">
-        <v>2677</v>
+        <v>2679</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>2181</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>2678</v>
+        <v>2680</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>2679</v>
+        <v>2681</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="4" t="s">
-        <v>2681</v>
+        <v>2683</v>
       </c>
       <c r="B91" s="4" t="s">
         <v>2197</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>2682</v>
+        <v>2684</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>2207</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>2683</v>
+        <v>2685</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="4" t="s">
-        <v>2684</v>
+        <v>2686</v>
       </c>
       <c r="B92" s="4" t="s">
         <v>2213</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>2685</v>
+        <v>2687</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>2223</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>2686</v>
+        <v>2688</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="4" t="s">
-        <v>2687</v>
+        <v>2689</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>2225</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>2688</v>
+        <v>2690</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>2231</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>2689</v>
+        <v>2691</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="4" t="s">
-        <v>2690</v>
+        <v>2692</v>
       </c>
       <c r="B94" s="4" t="s">
         <v>2237</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>2691</v>
+        <v>2693</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>2243</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>2236</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="4" t="s">
-        <v>2695</v>
+        <v>2697</v>
       </c>
       <c r="B95" s="4" t="s">
         <v>2245</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>2696</v>
+        <v>2698</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>2249</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>2244</v>
       </c>
       <c r="G95" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H95" s="4" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="4" t="s">
-        <v>2697</v>
+        <v>2699</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>2251</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>2698</v>
+        <v>2700</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>2252</v>
+        <v>2254</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="F96" s="4" t="s">
         <v>2250</v>
       </c>
       <c r="G96" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H96" s="4" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="4" t="s">
-        <v>2699</v>
+        <v>2701</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>2254</v>
+        <v>2256</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>2700</v>
+        <v>2702</v>
       </c>
       <c r="D97" s="4" t="s">
+        <v>2257</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>2694</v>
+      </c>
+      <c r="F97" s="4" t="s">
         <v>2255</v>
       </c>
-      <c r="E97" s="4" t="s">
-        <v>2692</v>
-      </c>
-      <c r="F97" s="4" t="s">
-        <v>2253</v>
-      </c>
       <c r="G97" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H97" s="4" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="4" t="s">
-        <v>2701</v>
+        <v>2703</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>2257</v>
+        <v>2259</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>2702</v>
+        <v>2704</v>
       </c>
       <c r="D98" s="4" t="s">
+        <v>2260</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>2694</v>
+      </c>
+      <c r="F98" s="4" t="s">
         <v>2258</v>
       </c>
-      <c r="E98" s="4" t="s">
-        <v>2692</v>
-      </c>
-      <c r="F98" s="4" t="s">
-        <v>2256</v>
-      </c>
       <c r="G98" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="4" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>2260</v>
+        <v>2262</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>2704</v>
+        <v>2706</v>
       </c>
       <c r="D99" s="4" t="s">
+        <v>2263</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>2694</v>
+      </c>
+      <c r="F99" s="4" t="s">
         <v>2261</v>
       </c>
-      <c r="E99" s="4" t="s">
-        <v>2692</v>
-      </c>
-      <c r="F99" s="4" t="s">
-        <v>2259</v>
-      </c>
       <c r="G99" s="4" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep achievement feedback readable under narrow zoom
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 14:55 BST</t>
+    <t>Snapshot: 07 September 2026, 15:01 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -188,7 +188,7 @@
     <t>Breadcrumbs and top toolbar</t>
   </si>
   <si>
-    <t>Nested course/record, club analytics and event parent links now retain exact IDs; breadcrumbs extracted into shared renderer and wrap with 44px parent links. Three breadcrumb unit tests pass; actual renderer fixture passes all six sizes (final-shared-browser.log).</t>
+    <t>Nested course/record, club analytics and event parent links now retain exact IDs; breadcrumbs extracted into shared renderer and wrap with 44px parent links. Three breadcrumb unit tests pass; actual renderer fixture passes all six sizes (final-shared-browser.log). Expanded shared-acceptance-final.log passes6.6s: keyboard focus pauses achievement dismissal beyond13s, six-size recovery/dedupe checks, two axe scans with zero violations, dark CSS200% zoom at1440/360 and explicit achievement internal-clipping checks. Native zoom remains distinct.</t>
   </si>
   <si>
     <t>Full application chrome/entity-label, screen-reader, zoom and theme matrix outstanding.</t>
@@ -383,7 +383,7 @@
     <t>Offline queue and sync status</t>
   </si>
   <si>
-    <t>Storage-error recovery and queued retry now have 44px targets; account-keyed state and request generation retained. Actual sync component with synthetic queue passes error→dead-letter recovery and owner switch at all six sizes (final-shared-browser.log).</t>
+    <t>Storage-error recovery and queued retry now have 44px targets; account-keyed state and request generation retained. Actual sync component with synthetic queue passes error→dead-letter recovery and owner switch at all six sizes (final-shared-browser.log). Expanded shared-acceptance-final.log passes6.6s: keyboard focus pauses achievement dismissal beyond13s, six-size recovery/dedupe checks, two axe scans with zero violations, dark CSS200% zoom at1440/360 and explicit achievement internal-clipping checks. Native zoom remains distinct.</t>
   </si>
   <si>
     <t>Real IndexedDB, service-worker replay, partial failure, reconnect and cross-account concurrency acceptance remains outstanding; fixture mock is not backend proof.</t>
@@ -401,10 +401,10 @@
     <t>Status labels and achievement feedback</t>
   </si>
   <si>
-    <t>Achievement dismiss target is 44px, long title/description and XP wrap. Actual provider fixture passes duplicate event dedupe, long text, manual dismissal and no overflow at all six sizes (final-shared-browser.log); 360 screenshot inspected.</t>
-  </si>
-  <si>
-    <t>Queued-toast limits, hover/focus timing, screen-reader announcement, native zoom and full theme acceptance outstanding.</t>
+    <t>Achievement dismiss target is 44px, long title/description and XP wrap. Actual provider fixture passes duplicate event dedupe, long text, manual dismissal and no overflow at all six sizes (final-shared-browser.log); 360 screenshot inspected. Expanded shared-acceptance-final.log passes6.6s: keyboard focus pauses achievement dismissal beyond13s, six-size recovery/dedupe checks, two axe scans with zero violations, dark CSS200% zoom at1440/360 and explicit achievement internal-clipping checks. Native zoom remains distinct.</t>
+  </si>
+  <si>
+    <t>Queued-toast limits, real screen-reader announcements, native zoom, physical safe areas and all theme/consumer acceptance remain outstanding. CSS zoom screenshot caught internal header/footer/tier clipping; fixed with wrapping and regression assertion, final screenshot inspected.</t>
   </si>
   <si>
     <t>Colour is not the only status signal, large numbers wrap safely and duplicate unlock notifications are prevented.</t>

</xml_diff>

<commit_message>
Align mobile route metadata with implemented companion pages
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 15:16 BST</t>
+    <t>Snapshot: 07 September 2026, 15:38 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -206,10 +206,10 @@
     <t>Account menu and surface switch</t>
   </si>
   <si>
-    <t>Explicit companion body visible at1440x900,1280x800,1024x800; fixed spacing roles and bottom clearance; native switch roundtrip retains query. G05-today-companion-* screenshots under output/playwright/ui-upgrade.</t>
-  </si>
-  <si>
-    <t>Companion body visible at390x844,360x800,1023x800; More switch preserves route/query; native links retain beforeunload support. Same G05 screenshot set and browser-final.log.</t>
+    <t>Explicit companion body visible at1440x900,1280x800,1024x800; fixed spacing roles and bottom clearance; native switch roundtrip retains query. G05-today-companion-* screenshots under output/playwright/ui-upgrade. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log).</t>
+  </si>
+  <si>
+    <t>Companion body visible at390x844,360x800,1023x800; More switch preserves route/query; native links retain beforeunload support. Same G05 screenshot set and browser-final.log. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log).</t>
   </si>
   <si>
     <t>Unsaved drafts on routes without DirtyFormBar, long account identity/avatar-error fixtures, full account action outcomes, screen-reader/zoom/theme checks outstanding. No new React Aria account adapter installed.</t>
@@ -230,10 +230,10 @@
     <t>Mobile bottom tabs and More navigation</t>
   </si>
   <si>
-    <t>Searchable More includes all authorised desktop canonical nav tasks plus Privacy; admin items use server role. Wide companion drawer bounded; 1440,1280,1024 browser search/empty/Escape-focus/44px target checks pass.</t>
-  </si>
-  <si>
-    <t>Same checks pass390x844,360x800,1023x800; five existing tabs preserved. G06-more-* screenshots under output/playwright/ui-upgrade. Unit tests verify player/admin navigation coverage and uniqueness.</t>
+    <t>Searchable More includes all authorised desktop canonical nav tasks plus Privacy; admin items use server role. Wide companion drawer bounded; 1440,1280,1024 browser search/empty/Escape-focus/44px target checks pass. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log).</t>
+  </si>
+  <si>
+    <t>Same checks pass390x844,360x800,1023x800; five existing tabs preserved. G06-more-* screenshots under output/playwright/ui-upgrade. Unit tests verify player/admin navigation coverage and uniqueness. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log).</t>
   </si>
   <si>
     <t>Many destination tasks still use mobile handoff/summary; this does not complete those tasks. 98-route destination/redirect audit, physical keyboard/safe-area, screen-reader, zoom and dark/contrast matrix remain outstanding.</t>
@@ -3095,10 +3095,10 @@
     <t>Score differential table</t>
   </si>
   <si>
-    <t>Actual owned fixture, both surfaces at 1440x900,1280x800,390x844,360x800,1023/1024: handicap-browser-wrapped.log PASS 21.9s. Full methods, nine-hole equivalents, incomplete-round exclusion, source details, tabs and no page overflow; 390 screenshot inspected. Fixed Score differentials saved-view destination from dead #rounds to canonical ?tab=rounds retaining query. Actual browser functional workflow passed1.5m all12contexts, including suggestionclick/URL/selectedtab and unchanged shot fields. However log contains Unexpected end of JSON input pageerror; existing test only logged errors. Tightened test to collect stacks/assert zero; rerun pending, no clean browser pass claimed.</t>
-  </si>
-  <si>
-    <t>Paid advanced Untitled compositions unavailable; accessible local composition. Full acceptance, screen reader, zoom, themes, permissions, large history and shared sticky-bar overlap outstanding. Round correction mutation unverified. Unexpected end of JSON input in actual browser run; strengthened no-error assertion and stack capture need rerun. See handicap-link-browser-final.log.</t>
+    <t>Actual owned fixture, both surfaces at 1440x900,1280x800,390x844,360x800,1023/1024: handicap-browser-wrapped.log PASS 21.9s. Full methods, nine-hole equivalents, incomplete-round exclusion, source details, tabs and no page overflow; 390 screenshot inspected. Fixed Score differentials saved-view destination from dead #rounds to canonical ?tab=rounds retaining query. Actual browser functional workflow passed1.5m all12contexts, including suggestionclick/URL/selectedtab and unchanged shot fields. However log contains Unexpected end of JSON input pageerror; existing test only logged errors. Tightened test to collect stacks/assert zero; rerun pending, no clean browser pass claimed. Strengthened rerun PASS29.1s with zero pageerrors, all12contexts and exact saved-view destination/query retained (handicap-link-no-errors.log).</t>
+  </si>
+  <si>
+    <t>Paid advanced Untitled compositions unavailable; accessible local composition. Full acceptance, screen reader, zoom, themes, permissions, large history and shared sticky-bar overlap outstanding. Round correction mutation unverified. Earlier intermittent JSON parse error did not reproduce in strengthened passing run; root cause unproven. No unchanged rerun needed.</t>
   </si>
   <si>
     <t>Nine-hole equivalents and fallback assumptions remain explicit.</t>

</xml_diff>

<commit_message>
Restore import preview views and fix modal club selection
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 17:00 BST</t>
+    <t>Snapshot: 07 September 2026, 17:08 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -317,10 +317,10 @@
     <t>Shared forms and confirmation behaviour</t>
   </si>
   <si>
-    <t>output/playwright/ui-upgrade/forms-browser.log:1passed11.2s all6sizes; confirmed native name/value, required validation, onClick, failed-save retention, focus/visible final field above footer; React Aria text/select/submit names and current value APIs. Full caller acceptance not claimed. Shared commit8a970995;151tests pass in isolated staged snapshot and types pass after Next typegen. PWA notice moved inside shell to avoid chrome overlap; initial queue loading distinguished from failure.</t>
-  </si>
-  <si>
-    <t>output/playwright/ui-upgrade/forms-browser.log:1passed11.2s all6sizes; confirmed native name/value, required validation, onClick, failed-save retention, focus/visible final field above footer; React Aria text/select/submit names and current value APIs. Full caller acceptance not claimed.</t>
+    <t>output/playwright/ui-upgrade/forms-browser.log:1passed11.2s all6sizes; confirmed native name/value, required validation, onClick, failed-save retention, focus/visible final field above footer; React Aria text/select/submit names and current value APIs. Full caller acceptance not claimed. Shared commit8a970995;151tests pass in isolated staged snapshot and types pass after Next typegen. PWA notice moved inside shell to avoid chrome overlap; initial queue loading distinguished from failure. 7 September import-view regression verified: local saved search/columns restore without navigation or lost corrections; complete filtered-batch CSV retained beyond20-row pagination. import-preview-controls-final.log passed8.1s at all six sizes, actual correction via React Aria picker, saved restore,25-row export from page2 and no errors/overflow. Found and fixed select popup blocked outside Radix modal by portalling inside closest dialog using installed Popover export. Actual import both surfaces/all sizes plus shared form regressions passed36.8s (import-preview-actual-and-forms.log). Types/lint pass; final360 screenshot inspected. Native AT/device and broader import acceptance remain open.</t>
+  </si>
+  <si>
+    <t>output/playwright/ui-upgrade/forms-browser.log:1passed11.2s all6sizes; confirmed native name/value, required validation, onClick, failed-save retention, focus/visible final field above footer; React Aria text/select/submit names and current value APIs. Full caller acceptance not claimed. 7 September import-view regression verified: local saved search/columns restore without navigation or lost corrections; complete filtered-batch CSV retained beyond20-row pagination. import-preview-controls-final.log passed8.1s at all six sizes, actual correction via React Aria picker, saved restore,25-row export from page2 and no errors/overflow. Found and fixed select popup blocked outside Radix modal by portalling inside closest dialog using installed Popover export. Actual import both surfaces/all sizes plus shared form regressions passed36.8s (import-preview-actual-and-forms.log). Types/lint pass; final360 screenshot inspected. Native AT/device and broader import acceptance remain open.</t>
   </si>
   <si>
     <t>Native and React Aria fixture passes; full caller draft/navigation, screenreader, theme/zoom and software-keyboard matrix outstanding. Paid modal code unavailable; accessible local Radix alternative registered.</t>
@@ -3260,7 +3260,7 @@
     <t>Shot preview and uncertain club review</t>
   </si>
   <si>
-    <t>All parsed shots retained with pagination/search; mobile detail sheet, warnings and source-row club corrections. UI-first batch: TypeScript/scoped lint pass; sample UI smoke1passed1.6m on both surfaces at1440x900,1280x800,390x844,360x800,1023x800,1024x800.5sample rows,disabled save,no pageerrors/no page overflow. Screenshots: output/playwright/ui-upgrade/import-ui-smoke. Mapping disclosure/quick-picker error display refined after smoke.</t>
+    <t>All parsed shots retained with pagination/search; mobile detail sheet, warnings and source-row club corrections. UI-first batch: TypeScript/scoped lint pass; sample UI smoke1passed1.6m on both surfaces at1440x900,1280x800,390x844,360x800,1023x800,1024x800.5sample rows,disabled save,no pageerrors/no page overflow. Screenshots: output/playwright/ui-upgrade/import-ui-smoke. Mapping disclosure/quick-picker error display refined after smoke. 7 September import-view regression verified: local saved search/columns restore without navigation or lost corrections; complete filtered-batch CSV retained beyond20-row pagination. import-preview-controls-final.log passed8.1s at all six sizes, actual correction via React Aria picker, saved restore,25-row export from page2 and no errors/overflow. Found and fixed select popup blocked outside Radix modal by portalling inside closest dialog using installed Popover export. Actual import both surfaces/all sizes plus shared form regressions passed36.8s (import-preview-actual-and-forms.log). Types/lint pass; final360 screenshot inspected. Native AT/device and broader import acceptance remain open.</t>
   </si>
   <si>
     <t>Unresolved club or unit ambiguity cannot be hidden by styling.</t>

</xml_diff>

<commit_message>
Integrate Today evidence workspace and measured highlight context
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 17:11 BST</t>
+    <t>Snapshot: 07 September 2026, 17:18 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -608,7 +608,7 @@
     <t>Today title and latest-session answer</t>
   </si>
   <si>
-    <t>Compact Today header, latest-session answer retained, extra hero heading changed to h2. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Compact Today header, latest-session answer retained, extra hero heading changed to h2. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>Today UI batch under final quick checks. Browser viewport/long/empty/loading/error/selection/action acceptance deferred to integration pass; no complete claim. One runtime JSON pageerror needs attribution/fix; native zoom/AT, complete correction and dynamic-state acceptance deferred. UI implemented does not mean accepted.</t>
@@ -626,7 +626,7 @@
     <t>Driver development summary on Today</t>
   </si>
   <si>
-    <t>Driver signal now context-dependent and disclosed below the main answer. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Driver signal now context-dependent and disclosed below the main answer. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>No contradiction with /speed or duplicated primary page title.</t>
@@ -641,7 +641,7 @@
     <t>Overview, Practice, Evidence and Data quality tabs</t>
   </si>
   <si>
-    <t>Controlled namespaced four-section tabs preserve URL query and mounted panel state; equivalent phone tasks added. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Controlled namespaced four-section tabs preserve URL query and mounted panel state; equivalent phone tasks added. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>All four content areas have a functional destination on both surfaces.</t>
@@ -656,7 +656,7 @@
     <t>Latest verdict, change and scoring trust</t>
   </si>
   <si>
-    <t>Existing verdict/scoring readouts retained with explicit directional limitation beside the affected evidence. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Existing verdict/scoring readouts retained with explicit directional limitation beside the affected evidence. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>A distance-valid but alignment-limited session keeps its valid distance evidence and warning.</t>
@@ -671,7 +671,7 @@
     <t>Shot patterns and dispersion</t>
   </si>
   <si>
-    <t>Original renderers retained; explicit shot selector complements plot interactions; mobile includes raw evidence with trust filtering. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Original renderers retained; explicit shot selector complements plot interactions; mobile includes raw evidence with trust filtering. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>Selected shot ID stays consistent across plot, table and rail.</t>
@@ -686,7 +686,7 @@
     <t>Selected shot details</t>
   </si>
   <si>
-    <t>Selected-shot source/history now reachable in bounded mobile drawer with visible close and shared review rail. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Selected-shot source/history now reachable in bounded mobile drawer with visible close and shared review rail. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>Missing measurements display as unavailable, never zero.</t>
@@ -701,7 +701,7 @@
     <t>Shot evidence and review actions</t>
   </si>
   <si>
-    <t>Phone selected-shot rail exposes reversible review and existing owner-scoped club correction; raw source preserved. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Phone selected-shot rail exposes reversible review and existing owner-scoped club correction; raw source preserved. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>Excluding is reversible, original data remains available and affected summaries refresh consistently.</t>
@@ -716,7 +716,7 @@
     <t>Alignment and data-quality checks</t>
   </si>
   <si>
-    <t>Session-specific alignment/direction warnings distinguish limited lateral evidence from valid carry/total/speed. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Session-specific alignment/direction warnings distinguish limited lateral evidence from valid carry/total/speed. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>Alignment concerns do not silently invalidate trustworthy carry or ball-speed data.</t>
@@ -731,7 +731,7 @@
     <t>Practice prescription, club performance and current loop</t>
   </si>
   <si>
-    <t>Existing plan/result and recommendation actions retained together in Practice; no new default drill. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement.</t>
+    <t>Existing plan/result and recommendation actions retained together in Practice; no new default drill. UI implementation applied; quick checks pending. UI smoke exercised both surfaces at 1440x900,1280x800,390x844,360x800,1023x800,1024x800: all four tabs, one h1, retained-panel visibility and no page overflow assertions passed; 12 screenshots in today-ui-ready. Overall smoke failed on one Unexpected end of JSON input pageerror; cause outstanding. Lint/types pass before final history/readiness refinement. 7 September reviewed coherent Today UI integration: shared four sections, full selected-shot review wiring, activity-vs-measured confidence labels, real handicap source/empty state, highlight source links and directional-quality context. today-integration-browser.log PASS24.4s both surfaces/all six sizes verifies section selection, single visible panel/heading and bounded layout;390 companion quality screenshot inspected. today-evidence-integration.log31PASS2.11s; finite highlight regression reproduced then fixed,16relatedtests PASS327ms. Types/scoped lint pass. This section smoke does not verify every correction/delete action or native AT/theme state.</t>
   </si>
   <si>
     <t>The CTA carries the same club/focus and uses saved evidence, not a generic default drill.</t>

</xml_diff>

<commit_message>
Avoid inferred source sessions in dashboard practice recommendations
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 17:18 BST</t>
+    <t>Snapshot: 07 September 2026, 17:22 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -746,7 +746,7 @@
     <t>Dashboard overview and priority</t>
   </si>
   <si>
-    <t>Compact full-width Dashboard with the same complete task and section links on both surfaces; removed phone redirect and desktop-only handoff. App smoke passed 11.2s: both surfaces at all six sizes, one h1, sections visible, no overflow/pageerrors; 12 screenshots dashboard-ui-smoke. Lint/types pass; 15 route/capability tests pass.</t>
+    <t>Compact full-width Dashboard with the same complete task and section links on both surfaces; removed phone redirect and desktop-only handoff. App smoke passed 11.2s: both surfaces at all six sizes, one h1, sections visible, no overflow/pageerrors; 12 screenshots dashboard-ui-smoke. Lint/types pass; 15 route/capability tests pass. 7 September Dashboard aggregate recommendation no longer attaches an inferred latest-session source. Club/source/time retained; saved plan branch unchanged. dashboard-practice-handoff.log PASS37.7s with older iron/newer Driver fixture, both surfaces/all six sizes, exact Practice arrival without sourceSessionId, original iron shot values unchanged, no errors/overflow. Scoped lint passed. This does not establish an exact evidence session for aggregate recommendations.</t>
   </si>
   <si>
     <t>Full keyboard/AT/native zoom, dynamic states and saved-plan/speed fixture consistency checks remain outstanding. Paid metrics example unavailable; local semantic metric composition registered. Browser smoke does not cover every interaction.</t>
@@ -779,7 +779,7 @@
     <t>Recommended practice</t>
   </si>
   <si>
-    <t>Saved plan ID or focused club/source-session practice handoff; specific drill/reason/duration/evidence. No fake completed balls or analytics link labelled Start. App smoke passed 11.2s: both surfaces at all six sizes, one h1, sections visible, no overflow/pageerrors; 12 screenshots dashboard-ui-smoke. Lint/types pass; 15 route/capability tests pass.</t>
+    <t>Saved plan ID or focused club/source-session practice handoff; specific drill/reason/duration/evidence. No fake completed balls or analytics link labelled Start. App smoke passed 11.2s: both surfaces at all six sizes, one h1, sections visible, no overflow/pageerrors; 12 screenshots dashboard-ui-smoke. Lint/types pass; 15 route/capability tests pass. 7 September Dashboard aggregate recommendation no longer attaches an inferred latest-session source. Club/source/time retained; saved plan branch unchanged. dashboard-practice-handoff.log PASS37.7s with older iron/newer Driver fixture, both surfaces/all six sizes, exact Practice arrival without sourceSessionId, original iron shot values unchanged, no errors/overflow. Scoped lint passed. This does not establish an exact evidence session for aggregate recommendations.</t>
   </si>
   <si>
     <t>Starting the plan retains its specific target and evidence context.</t>

</xml_diff>

<commit_message>
Restore shared session views and preserve finite owner metrics
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 17:22 BST</t>
+    <t>Snapshot: 07 September 2026, 17:35 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -233,7 +233,7 @@
     <t>Searchable More includes all authorised desktop canonical nav tasks plus Privacy; admin items use server role. Wide companion drawer bounded; 1440,1280,1024 browser search/empty/Escape-focus/44px target checks pass. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log).</t>
   </si>
   <si>
-    <t>Same checks pass390x844,360x800,1023x800; five existing tabs preserved. G06-more-* screenshots under output/playwright/ui-upgrade. Unit tests verify player/admin navigation coverage and uniqueness. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log).</t>
+    <t>Same checks pass390x844,360x800,1023x800; five existing tabs preserved. G06-more-* screenshots under output/playwright/ui-upgrade. Unit tests verify player/admin navigation coverage and uniqueness. Canonical mobileExperience metadata reconciled to implemented companion routes; hidden/admin nav remains hidden, permissions unchanged, unknown nested handoffs retained. Twenty route metadata/gate tests pass1.51s; types/lint pass (route-metadata-alignment.log). 2026-09-07 shared-account browser verifies bounded long compact title after w-full/max-w-full fix; screenshot no longer overlaps navigation controls.</t>
   </si>
   <si>
     <t>Many destination tasks still use mobile handoff/summary; this does not complete those tasks. 98-route destination/redirect audit, physical keyboard/safe-area, screen-reader, zoom and dark/contrast matrix remain outstanding.</t>
@@ -5666,13 +5666,13 @@
     <t>Shared player identity and role context</t>
   </si>
   <si>
-    <t>One shared identity/read-only role context, full scoped metrics, loaded20 session search/order and semantic table. Types shared-account-types.log/scopedlint clean. Backend shared-account-data-final.log1PASS1.14s: all3roles/owner, revoked/noaccess/invalidUUID, owner-only eligible distance, minimalprofile projection and partialscore null.</t>
-  </si>
-  <si>
-    <t>Same complete shared task on both surfaces, full session details in responsive panel including course/source/date/type/score/holes; safe account-unavailable route. Actual shared-account-browser-final.logFAILED before page: surface/workbench500 Unexpected end of JSON input in runtime. No viewport pass claimed.</t>
-  </si>
-  <si>
-    <t>Actual12surface/viewport UI, screenshot/focus/keyboard, all empty/error/AT/zoom/theme states outstanding due local runtime JSONparsefailure before route. First fixture missing raw_csv_text corrected; not runtime defect. Latest20 remains disclosed loaded limit, no serverpagination added. No session deep links because target owner-only routes do not establish shared access. Paid metrics/table templates unavailable; semantic local alternatives.</t>
+    <t>One shared identity/read-only role context, full scoped metrics, loaded20 session search/order and semantic table. Types shared-account-types.log/scopedlint clean. Backend shared-account-data-final.log1PASS1.14s: all3roles/owner, revoked/noaccess/invalidUUID, owner-only eligible distance, minimalprofile projection and partialscore null. 2026-09-07: shared-ledger-controls-final.log PASS1.4m on both surfaces at all six required sizes: search/date order, filtered CSV contents and hidden headers, saved-view restore and reload persistence, complete/partial drawer fields, foreign-owner exclusion and actual membership revocation. Long mobile title bounds repaired; 390px companion controls screenshot inspected. Types and scoped lint clean. shared-finite-fixed.log2DB tests PASS2.69s: longest total excludes NaN/Infinity/nonpositive without discarding shot counts.</t>
+  </si>
+  <si>
+    <t>Same complete shared task on both surfaces, full session details in responsive panel including course/source/date/type/score/holes; safe account-unavailable route. Actual shared-account-browser-final.logFAILED before page: surface/workbench500 Unexpected end of JSON input in runtime. No viewport pass claimed. 2026-09-07: shared-ledger-controls-final.log PASS1.4m on both surfaces at all six required sizes: search/date order, filtered CSV contents and hidden headers, saved-view restore and reload persistence, complete/partial drawer fields, foreign-owner exclusion and actual membership revocation. Long mobile title bounds repaired; 390px companion controls screenshot inspected. Types and scoped lint clean. shared-finite-fixed.log2DB tests PASS2.69s: longest total excludes NaN/Infinity/nonpositive without discarding shot counts.</t>
+  </si>
+  <si>
+    <t>Earlier local JSONparse failure is historical; current twelve-variant browser run passes. Native AT/device/zoom/theme and full empty/error matrix remain outstanding. Latest20 loaded limit remains disclosed; no server pagination. Paid templates unavailable; accessible local composition. No shared owner-only deep links or mutation permissions added.</t>
   </si>
   <si>
     <t>This route does not impersonate the owner or turn a read-only overview into mutation access.</t>
@@ -5699,7 +5699,7 @@
     <t>Unauthorised or revoked access returns an explicit safe state.</t>
   </si>
   <si>
-    <t>src/app/(app)/shared/[userId]/page.tsx; src/components/ui/table.tsx</t>
+    <t>src/app/(app)/shared/[userId]/page.tsx; src/components/ui/table.tsx; src/app/shared/shared-session-ledger.tsx</t>
   </si>
   <si>
     <t>P75-C01</t>

</xml_diff>

<commit_message>
Restore a complete independent mobile shared scorecard
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 17:35 BST</t>
+    <t>Snapshot: 07 September 2026, 17:39 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6635,13 +6635,13 @@
     <t>Shared round identity and scope</t>
   </si>
   <si>
-    <t>Both surfaces reuse full public scorecard, named owner/date/current limited scope, recorded partial counts/totals, row headers and pinned identity. Differential hidden unless valid complete9/18card; calculation unchanged. Dedicated safe404/loading/error recovery. shared-round-browser.log1PASS6.5s all12 surface/viewports,18rows/manualputts/fullrounddetails/read-only/noindex/nooverflow/noerrors; revocation removes data. Types/lint pass.</t>
-  </si>
-  <si>
-    <t>Same complete labelled horizontal scorecard with pinned hole identity and all existing allowed fields, full round details and public navigation.390/360/1023 checked on both surfaces;390 screenshot inspected. No private-app controls.</t>
-  </si>
-  <si>
-    <t>Backend DTO still calculates differential for partial cards; presentation suppression is not service fix (shared-round-partial.test.ts documented intentional failure). Full complete/empty/malformed/service-error browser matrix, keyboard table scroll, screen reader/native zoom/themes/physical touch outstanding. Access backend test separately verifies expired/revoked/wrong owner. Paid advanced examples unavailable; local semantic alternatives.</t>
+    <t>Both surfaces reuse full public scorecard, named owner/date/current limited scope, recorded partial counts/totals, row headers and pinned identity. Differential hidden unless valid complete9/18card; calculation unchanged. Dedicated safe404/loading/error recovery. shared-round-browser.log1PASS6.5s all12 surface/viewports,18rows/manualputts/fullrounddetails/read-only/noindex/nooverflow/noerrors; revocation removes data. Types/lint pass. 2026-09-07: shared-round-companion-native.log PASS6.2s both surfaces x six required sizes, complete permitted18-hole fields/manual-putt labels, partial score/no differential, native round-details disclosure, keyboard table scroll, no overflow/page errors, no edit/delete controls, noindex and actual revoked-link rejection. Companion uses independent native pinned-identity table instead of importing workbench. Four graph/security source checks PASS; scoped lint/types clean. 360px screenshot inspected.</t>
+  </si>
+  <si>
+    <t>Same complete labelled horizontal scorecard with pinned hole identity and all existing allowed fields, full round details and public navigation.390/360/1023 checked on both surfaces;390 screenshot inspected. No private-app controls. 2026-09-07: shared-round-companion-native.log PASS6.2s both surfaces x six required sizes, complete permitted18-hole fields/manual-putt labels, partial score/no differential, native round-details disclosure, keyboard table scroll, no overflow/page errors, no edit/delete controls, noindex and actual revoked-link rejection. Companion uses independent native pinned-identity table instead of importing workbench. Four graph/security source checks PASS; scoped lint/types clean. 360px screenshot inspected.</t>
+  </si>
+  <si>
+    <t>Backend DTO still calculates differential for partial cards; presentation suppression is not service fix (shared-round-partial.test.ts documented intentional failure). Full complete/empty/malformed/service-error browser matrix, keyboard table scroll, screen reader/native zoom/themes/physical touch outstanding. Access backend test separately verifies expired/revoked/wrong owner. Paid advanced examples unavailable; local semantic alternatives. Native device/AT/theme and comprehensive expired/empty/error fixtures remain outstanding. Earlier public-wide companion visibility and early disclosure click failures repaired before final passing run. Paid table template remains unavailable; local semantic table alternative.</t>
   </si>
   <si>
     <t>Only the token-authorised frozen/current scope supported by the existing link is exposed.</t>

</xml_diff>

<commit_message>
Add golf imagery and subtle card gradients to Analyse
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 17:52 BST</t>
+    <t>Snapshot: 07 September 2026, 17:54 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -2147,10 +2147,10 @@
     <t>Analysis title and evidence overview</t>
   </si>
   <si>
-    <t>Analysis workbench browser passed13.8s at1440x900,1280x800,390x844,360x800,1023x800,1024x800: compact title, provenance open/close/repair, illustrative SVG label, scoped comparison link, one h1/no page overflow. analyse-ui-smoke.log; TypeScript/scoped lint passed.</t>
-  </si>
-  <si>
-    <t>Both-surface six-size hub browser passed in analysis-workspace-hub-browser.log after mobile Compare sessions/Conditions/Analysis workspace destinations implemented. Provenance open/close/repair, illustrative SVG label, scope links, one h1/no overflow. P22 companion screenshots available.</t>
+    <t>Analysis workbench browser passed13.8s at1440x900,1280x800,390x844,360x800,1023x800,1024x800: compact title, provenance open/close/repair, illustrative SVG label, scoped comparison link, one h1/no page overflow. analyse-ui-smoke.log; TypeScript/scoped lint passed. 2026-09-07 user-requested visual refinement: existing golf image in Analysis hero with dark readable overlay and responsive Next Image; subtle scoped gradients on insight/conditions/quality cards. analyse-atmosphere.log PASS34.9s both surfaces x six sizes, image actually loaded, no page overflow and provenance drawer/links retained. 1440desktop and360mobile screenshots visually inspected; types/lint clean. Decorative image has empty alt and does not represent measured shot evidence.</t>
+  </si>
+  <si>
+    <t>Both-surface six-size hub browser passed in analysis-workspace-hub-browser.log after mobile Compare sessions/Conditions/Analysis workspace destinations implemented. Provenance open/close/repair, illustrative SVG label, scope links, one h1/no overflow. P22 companion screenshots available. 2026-09-07 user-requested visual refinement: existing golf image in Analysis hero with dark readable overlay and responsive Next Image; subtle scoped gradients on insight/conditions/quality cards. analyse-atmosphere.log PASS34.9s both surfaces x six sizes, image actually loaded, no page overflow and provenance drawer/links retained. 1440desktop and360mobile screenshots visually inspected; types/lint clean. Decorative image has empty alt and does not represent measured shot evidence.</t>
   </si>
   <si>
     <t>Full destination task acceptance, state/AT/zoom/theme verification outstanding. Existing trusted-evidence date range mixes overall earliest session with latest trusted session; review scope reconciliation before acceptance. No paid component entitlement claimed.</t>

</xml_diff>

<commit_message>
Integrate UI upgrade and preserve outstanding acceptance evidence
</commit_message>
<xml_diff>
--- a/ForeKingHell-completion-tracker.xlsx
+++ b/ForeKingHell-completion-tracker.xlsx
@@ -26,7 +26,7 @@
     <t>ForeKingHell · UI upgrade progress</t>
   </si>
   <si>
-    <t>Snapshot: 07 September 2026, 18:56 BST</t>
+    <t>Snapshot: 07 September 2026, 19:06 BST</t>
   </si>
   <si>
     <t>UI-first delivery: implemented UI is shown first below. Acceptance is tracked separately and remains pending until its checks pass. Filter Components or open Work touched for the exact changes and evidence. Source: ForeKingHell-completion-tracker.csv.</t>
@@ -6152,10 +6152,10 @@
     <t>Health register</t>
   </si>
   <si>
-    <t>Full shared health summary/register with priority/search/result controls and complete diagnostics. Actual recorded DB check reviewed then saved to dated audit history; provider health remains unknown. admin-system-browser.log 1 passed35.7s both surfaces/all6; confirmed refresh adds exact one audit and previous seven-failure snapshot retained. Types/scoped lint clean. Follow-up: restored shared saved views, filtered CSV export and column controls with URL-backed health filters/order. Scoped lint passed; new control browser readback outstanding with verification agent. Not in hosted preview.</t>
-  </si>
-  <si>
-    <t>390x844,360x800,1023x800,1024x800 complete diagnostics, Cancel/no write, exact recorded refresh and native expandable chronological history; no overflow/pageerrors. Companion390 screenshot inspected. Follow-up: restored shared saved views, filtered CSV export and column controls with URL-backed health filters/order. Scoped lint passed; new control browser readback outstanding with verification agent. Not in hosted preview.</t>
+    <t>Full shared health summary/register with priority/search/result controls and complete diagnostics. Actual recorded DB check reviewed then saved to dated audit history; provider health remains unknown. admin-system-browser.log 1 passed35.7s both surfaces/all6; confirmed refresh adds exact one audit and previous seven-failure snapshot retained. Types/scoped lint clean. Follow-up: restored shared saved views, filtered CSV export and column controls with URL-backed health filters/order. Scoped lint passed; new control browser readback outstanding with verification agent. Not in hosted preview. Follow-up verification PASS: admin-system-restored-retry.log 1.4m, both surfaces/six sizes, filtered CSV excludes other checks and hidden timestamp, saved view restores filters/columns through reload. Earlier pending readback resolved; broader acceptance remains partial.</t>
+  </si>
+  <si>
+    <t>390x844,360x800,1023x800,1024x800 complete diagnostics, Cancel/no write, exact recorded refresh and native expandable chronological history; no overflow/pageerrors. Companion390 screenshot inspected. Follow-up: restored shared saved views, filtered CSV export and column controls with URL-backed health filters/order. Scoped lint passed; new control browser readback outstanding with verification agent. Not in hosted preview. Follow-up verification PASS: admin-system-restored-retry.log 1.4m, both surfaces/six sizes, filtered CSV excludes other checks and hidden timestamp, saved view restores filters/columns through reload. Earlier pending readback resolved; broader acceptance remains partial.</t>
   </si>
   <si>
     <t>Sensitive operational information remains admin-only.</t>

</xml_diff>